<commit_message>
Ausführen des Create Context Connections Skripts
</commit_message>
<xml_diff>
--- a/context_connections.xlsx
+++ b/context_connections.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofcambridgecloud-my.sharepoint.com/personal/lf576_cam_ac_uk/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofcambridgecloud-my.sharepoint.com/personal/lf576_cam_ac_uk/Documents/04_Coding/hydrogenation/current_versions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C5C5D99A-F90E-4DDA-B551-364ECC0B9EB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{C5C5D99A-F90E-4DDA-B551-364ECC0B9EB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47D2A7D8-5825-4BBE-8ADB-80B48ACFF74A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{2AABB6A2-CE1B-404B-9F86-D510FD910096}"/>
   </bookViews>
@@ -53,9 +53,6 @@
     <t>Space</t>
   </si>
   <si>
-    <t>Stucture</t>
-  </si>
-  <si>
     <t>Substance</t>
   </si>
   <si>
@@ -123,6 +120,9 @@
   </si>
   <si>
     <t>#InitialVolume_LiquidPhase</t>
+  </si>
+  <si>
+    <t>Structure</t>
   </si>
 </sst>
 </file>
@@ -183,6 +183,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -504,6 +508,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED4507CF-D6FB-4A2B-A3A9-62CC9ECEF7FC}">
   <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.28515625" customWidth="1"/>
+    <col min="2" max="2" width="43.5703125" customWidth="1"/>
+    <col min="3" max="3" width="30.28515625" customWidth="1"/>
+    <col min="4" max="4" width="26.28515625" customWidth="1"/>
+    <col min="5" max="5" width="29" customWidth="1"/>
+    <col min="6" max="6" width="19.42578125" customWidth="1"/>
+    <col min="7" max="7" width="23.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
@@ -519,118 +532,118 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" t="s">
         <v>4</v>
-      </c>
-      <c r="G1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>11</v>
-      </c>
-      <c r="D3" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
         <v>13</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>14</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" t="s">
         <v>17</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>18</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>19</v>
-      </c>
-      <c r="D6" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D7" s="1"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
         <v>22</v>
       </c>
-      <c r="C8" t="s">
+      <c r="E8" t="s">
         <v>23</v>
-      </c>
-      <c r="E8" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Umwandeln der Contextbezeichnungen von xxxInformation zu xxx_Information
</commit_message>
<xml_diff>
--- a/context_connections.xlsx
+++ b/context_connections.xlsx
@@ -8,16 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofcambridgecloud-my.sharepoint.com/personal/lf576_cam_ac_uk/Documents/04_Coding/hydrogenation/current_versions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="8_{C5C5D99A-F90E-4DDA-B551-364ECC0B9EB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0522EE5F-A51E-43D9-80CD-FBA415E9F6E8}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="8_{C5C5D99A-F90E-4DDA-B551-364ECC0B9EB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E30796E9-3E09-428C-9C07-8712B9CE6741}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{2AABB6A2-CE1B-404B-9F86-D510FD910096}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2AABB6A2-CE1B-404B-9F86-D510FD910096}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,30 +38,8 @@
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="103">
   <si>
     <t>Information</t>
   </si>
@@ -85,6 +60,294 @@
   </si>
   <si>
     <t>Entity</t>
+  </si>
+  <si>
+    <t>#Reactor</t>
+  </si>
+  <si>
+    <t>#DigitalObjectID_Reactor</t>
+  </si>
+  <si>
+    <t>#TemperatureSensor_Energy</t>
+  </si>
+  <si>
+    <t>#LastUsedTime_Reactor</t>
+  </si>
+  <si>
+    <t>#LastUsedPurpose_Reactor_BeforeFirstUse</t>
+  </si>
+  <si>
+    <t>#PressureSensor_Energy</t>
+  </si>
+  <si>
+    <t>#LastServicedTime_Reactor</t>
+  </si>
+  <si>
+    <t>#OperatingMode_Reactor</t>
+  </si>
+  <si>
+    <t>#SetPressureProfile_Reactor</t>
+  </si>
+  <si>
+    <t>#ExperimentalProcedure</t>
+  </si>
+  <si>
+    <t>#SetTemperatureProfile_Reactor</t>
+  </si>
+  <si>
+    <t>#Vessel</t>
+  </si>
+  <si>
+    <t>#DigitalObjectID_Vessel</t>
+  </si>
+  <si>
+    <t>#Reactor_Energy</t>
+  </si>
+  <si>
+    <t>#LastUsedTime_Vessel</t>
+  </si>
+  <si>
+    <t>#LastUsedPurpose_Vessel_BeforeFirstUse</t>
+  </si>
+  <si>
+    <t>#Reactor_Time</t>
+  </si>
+  <si>
+    <t>#Stirrer</t>
+  </si>
+  <si>
+    <t>#DigitalObjectID_Stirrer</t>
+  </si>
+  <si>
+    <t>#LastUsedTime_Stirrer</t>
+  </si>
+  <si>
+    <t>#LastUsedPurpose_Stirrer_BeforeFirstUse</t>
+  </si>
+  <si>
+    <t>#SetRPMProfile_Reactor</t>
+  </si>
+  <si>
+    <t>#Sparger</t>
+  </si>
+  <si>
+    <t>#DigitalObjectID_Sparger</t>
+  </si>
+  <si>
+    <t>#LastUsedTime_Sparger</t>
+  </si>
+  <si>
+    <t>#LastUsedPurpose_Sparger_BeforeFirstUse</t>
+  </si>
+  <si>
+    <t>#SetPressureProfile_Sparger</t>
+  </si>
+  <si>
+    <t>#Jacket</t>
+  </si>
+  <si>
+    <t>#DigitalObjectID_Jacket</t>
+  </si>
+  <si>
+    <t>#LastUsedTime_Jacket</t>
+  </si>
+  <si>
+    <t>#LastUsedPurpose_Jacket_BeforeFirstUse</t>
+  </si>
+  <si>
+    <t>#SetFlowrateProfile_Jacket</t>
+  </si>
+  <si>
+    <t>#TemperatureSensor</t>
+  </si>
+  <si>
+    <t>#LastUsedPurpose_TemperatureSensor_BeforeFirstUse</t>
+  </si>
+  <si>
+    <t>#DigitalObjectID_TemperatureSensor</t>
+  </si>
+  <si>
+    <t>#RecordedTemperature_Reactor</t>
+  </si>
+  <si>
+    <t>#LastUsedTime_TemperatureSensor</t>
+  </si>
+  <si>
+    <t>#PressureSensor</t>
+  </si>
+  <si>
+    <t>#LastUsedPurpose_PressureSensor_BeforeFirstUse</t>
+  </si>
+  <si>
+    <t>#DigitalObjectID_PressureSensor</t>
+  </si>
+  <si>
+    <t>#RecordedPressure_Reactor</t>
+  </si>
+  <si>
+    <t>#LastUsedTime_PressureSensor</t>
+  </si>
+  <si>
+    <t>#MassFlowMeter</t>
+  </si>
+  <si>
+    <t>#LastUsedPurpose_MassFlowMeter_BeforeFirstUse</t>
+  </si>
+  <si>
+    <t>#DigitalObjectID_MassFlowMeter</t>
+  </si>
+  <si>
+    <t>#UsedGasVolume_H2</t>
+  </si>
+  <si>
+    <t>#LastUsedTime_MassFlowMeter</t>
+  </si>
+  <si>
+    <t>#Balance</t>
+  </si>
+  <si>
+    <t>#LastUsedPurpose_Balance_BeforeFirstUse</t>
+  </si>
+  <si>
+    <t>#LastUsedTime_Balance</t>
+  </si>
+  <si>
+    <t>#DigitalObjectID_Balance</t>
+  </si>
+  <si>
+    <t>#LiquidPhase</t>
+  </si>
+  <si>
+    <t>#Vessel_Energy</t>
+  </si>
+  <si>
+    <t>#Vessel_Space</t>
+  </si>
+  <si>
+    <t>#InitialMassFraction_Solvent_LiquidPhase</t>
+  </si>
+  <si>
+    <t>#Vessel_Structure</t>
+  </si>
+  <si>
+    <t>#InitialMassFraction_Water_LiquidPhase</t>
+  </si>
+  <si>
+    <t>#MaterialVolume_Reactor</t>
+  </si>
+  <si>
+    <t>#InitialVolume_LiquidPhase</t>
+  </si>
+  <si>
+    <t>#SolidPhase</t>
+  </si>
+  <si>
+    <t>#RDY_Energy</t>
+  </si>
+  <si>
+    <t>#CatalystPhase</t>
+  </si>
+  <si>
+    <t>#GasPhase</t>
+  </si>
+  <si>
+    <t>#DispersedGasPhase</t>
+  </si>
+  <si>
+    <t>#CoolingFluidPhase</t>
+  </si>
+  <si>
+    <t>#Jacket_Energy</t>
+  </si>
+  <si>
+    <t>#Jacket_Space</t>
+  </si>
+  <si>
+    <t>#Jacket_Structure</t>
+  </si>
+  <si>
+    <t>#CoolingFluidStream</t>
+  </si>
+  <si>
+    <t>#HydrogenSpargerPhase</t>
+  </si>
+  <si>
+    <t>#Sparger_Energy</t>
+  </si>
+  <si>
+    <t>#Sparger_Space</t>
+  </si>
+  <si>
+    <t>#Sparger_Structure</t>
+  </si>
+  <si>
+    <t>#HydrogenStream</t>
+  </si>
+  <si>
+    <t>#CleaningFluidPhase</t>
+  </si>
+  <si>
+    <t>#H2</t>
+  </si>
+  <si>
+    <t>#GasPhase_Energy</t>
+  </si>
+  <si>
+    <t>#H3</t>
+  </si>
+  <si>
+    <t>#DispersedGasPhase_Energy</t>
+  </si>
+  <si>
+    <t>#H4</t>
+  </si>
+  <si>
+    <t>#HydrogenSpargerPhase_Energy</t>
+  </si>
+  <si>
+    <t>#H2O</t>
+  </si>
+  <si>
+    <t>#LiquidPhase_Energy</t>
+  </si>
+  <si>
+    <t>#LiquidPhase_Space</t>
+  </si>
+  <si>
+    <t>#Solvent</t>
+  </si>
+  <si>
+    <t>#RDY</t>
+  </si>
+  <si>
+    <t>#SolidPhase_Energy</t>
+  </si>
+  <si>
+    <t>#StartMass_RDY</t>
+  </si>
+  <si>
+    <t>#FinalMass_RDY</t>
+  </si>
+  <si>
+    <t>#RDEt</t>
+  </si>
+  <si>
+    <t>#FinalMassRDEt</t>
+  </si>
+  <si>
+    <t>#Dimer1</t>
+  </si>
+  <si>
+    <t>#FinalMass_Dimer</t>
+  </si>
+  <si>
+    <t>#Dimer2</t>
+  </si>
+  <si>
+    <t>#Pt</t>
+  </si>
+  <si>
+    <t>#CatalystPhase_Energy</t>
   </si>
 </sst>
 </file>
@@ -137,625 +400,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Instructions"/>
-      <sheetName val="Overview"/>
-      <sheetName val="CaseStudy_Hydrogenation"/>
-      <sheetName val="Context_Hydrogenation_New"/>
-      <sheetName val="Context_Compact"/>
-      <sheetName val="Context Hydrogenation"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3">
-        <row r="4">
-          <cell r="A4" t="str">
-            <v>#Reactor</v>
-          </cell>
-          <cell r="B4" t="str">
-            <v>#DigitalObjectID_Reactor</v>
-          </cell>
-          <cell r="C4" t="str">
-            <v>#TemperatureSensor_Energy</v>
-          </cell>
-          <cell r="D4" t="str">
-            <v>#LastUsedTime_Reactor</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5" t="str">
-            <v>#Reactor</v>
-          </cell>
-          <cell r="B5" t="str">
-            <v>#LastUsedPurpose_Reactor_BeforeFirstUse</v>
-          </cell>
-          <cell r="C5" t="str">
-            <v>#PressureSensor_Energy</v>
-          </cell>
-          <cell r="D5" t="str">
-            <v>#LastServicedTime_Reactor</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6" t="str">
-            <v>#Reactor</v>
-          </cell>
-          <cell r="B6" t="str">
-            <v>#OperatingMode_Reactor</v>
-          </cell>
-          <cell r="C6" t="str">
-            <v>#SetPressureProfile_Reactor</v>
-          </cell>
-          <cell r="D6" t="str">
-            <v>#ExperimentalProcedure</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7" t="str">
-            <v>#Reactor</v>
-          </cell>
-          <cell r="C7" t="str">
-            <v>#SetTemperatureProfile_Reactor</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="A16" t="str">
-            <v>#Vessel</v>
-          </cell>
-          <cell r="B16" t="str">
-            <v>#DigitalObjectID_Vessel</v>
-          </cell>
-          <cell r="C16" t="str">
-            <v>#Reactor_Energy</v>
-          </cell>
-          <cell r="D16" t="str">
-            <v>#LastUsedTime_Vessel</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="A17" t="str">
-            <v>#Vessel</v>
-          </cell>
-          <cell r="B17" t="str">
-            <v>#LastUsedPurpose_Vessel_BeforeFirstUse</v>
-          </cell>
-          <cell r="D17" t="str">
-            <v>#Reactor_Time</v>
-          </cell>
-        </row>
-        <row r="29">
-          <cell r="A29" t="str">
-            <v>#Stirrer</v>
-          </cell>
-          <cell r="B29" t="str">
-            <v>#DigitalObjectID_Stirrer</v>
-          </cell>
-          <cell r="C29" t="str">
-            <v>#Reactor_Energy</v>
-          </cell>
-          <cell r="D29" t="str">
-            <v>#LastUsedTime_Stirrer</v>
-          </cell>
-        </row>
-        <row r="30">
-          <cell r="A30" t="str">
-            <v>#Stirrer</v>
-          </cell>
-          <cell r="B30" t="str">
-            <v>#LastUsedPurpose_Stirrer_BeforeFirstUse</v>
-          </cell>
-          <cell r="C30" t="str">
-            <v>#SetRPMProfile_Reactor</v>
-          </cell>
-          <cell r="D30" t="str">
-            <v>#Reactor_Time</v>
-          </cell>
-        </row>
-        <row r="42">
-          <cell r="A42" t="str">
-            <v>#Sparger</v>
-          </cell>
-          <cell r="B42" t="str">
-            <v>#DigitalObjectID_Sparger</v>
-          </cell>
-          <cell r="C42" t="str">
-            <v>#Reactor_Energy</v>
-          </cell>
-          <cell r="D42" t="str">
-            <v>#LastUsedTime_Sparger</v>
-          </cell>
-        </row>
-        <row r="43">
-          <cell r="A43" t="str">
-            <v>#Sparger</v>
-          </cell>
-          <cell r="B43" t="str">
-            <v>#LastUsedPurpose_Sparger_BeforeFirstUse</v>
-          </cell>
-          <cell r="C43" t="str">
-            <v>#SetPressureProfile_Sparger</v>
-          </cell>
-          <cell r="D43" t="str">
-            <v>#Reactor_Time</v>
-          </cell>
-        </row>
-        <row r="55">
-          <cell r="A55" t="str">
-            <v>#Jacket</v>
-          </cell>
-          <cell r="B55" t="str">
-            <v>#DigitalObjectID_Jacket</v>
-          </cell>
-          <cell r="C55" t="str">
-            <v>#Reactor_Energy</v>
-          </cell>
-          <cell r="D55" t="str">
-            <v>#LastUsedTime_Jacket</v>
-          </cell>
-        </row>
-        <row r="56">
-          <cell r="A56" t="str">
-            <v>#Jacket</v>
-          </cell>
-          <cell r="B56" t="str">
-            <v>#LastUsedPurpose_Jacket_BeforeFirstUse</v>
-          </cell>
-          <cell r="C56" t="str">
-            <v>#SetFlowrateProfile_Jacket</v>
-          </cell>
-          <cell r="D56" t="str">
-            <v>#Reactor_Time</v>
-          </cell>
-        </row>
-        <row r="68">
-          <cell r="A68" t="str">
-            <v>#TemperatureSensor</v>
-          </cell>
-          <cell r="B68" t="str">
-            <v>#LastUsedPurpose_TemperatureSensor_BeforeFirstUse</v>
-          </cell>
-          <cell r="C68" t="str">
-            <v>#Reactor_Energy</v>
-          </cell>
-          <cell r="D68" t="str">
-            <v>#Reactor_Time</v>
-          </cell>
-        </row>
-        <row r="69">
-          <cell r="A69" t="str">
-            <v>#TemperatureSensor</v>
-          </cell>
-          <cell r="B69" t="str">
-            <v>#DigitalObjectID_TemperatureSensor</v>
-          </cell>
-          <cell r="C69" t="str">
-            <v>#RecordedTemperature_Reactor</v>
-          </cell>
-          <cell r="D69" t="str">
-            <v>#LastUsedTime_TemperatureSensor</v>
-          </cell>
-        </row>
-        <row r="81">
-          <cell r="A81" t="str">
-            <v>#PressureSensor</v>
-          </cell>
-          <cell r="B81" t="str">
-            <v>#LastUsedPurpose_PressureSensor_BeforeFirstUse</v>
-          </cell>
-          <cell r="C81" t="str">
-            <v>#Reactor_Energy</v>
-          </cell>
-          <cell r="D81" t="str">
-            <v>#Reactor_Time</v>
-          </cell>
-        </row>
-        <row r="82">
-          <cell r="A82" t="str">
-            <v>#PressureSensor</v>
-          </cell>
-          <cell r="B82" t="str">
-            <v>#DigitalObjectID_PressureSensor</v>
-          </cell>
-          <cell r="C82" t="str">
-            <v>#RecordedPressure_Reactor</v>
-          </cell>
-          <cell r="D82" t="str">
-            <v>#LastUsedTime_PressureSensor</v>
-          </cell>
-        </row>
-        <row r="94">
-          <cell r="A94" t="str">
-            <v>#MassFlowMeter</v>
-          </cell>
-          <cell r="B94" t="str">
-            <v>#LastUsedPurpose_MassFlowMeter_BeforeFirstUse</v>
-          </cell>
-          <cell r="C94" t="str">
-            <v>#Reactor_Energy</v>
-          </cell>
-          <cell r="D94" t="str">
-            <v>#Reactor_Time</v>
-          </cell>
-        </row>
-        <row r="95">
-          <cell r="A95" t="str">
-            <v>#MassFlowMeter</v>
-          </cell>
-          <cell r="B95" t="str">
-            <v>#DigitalObjectID_MassFlowMeter</v>
-          </cell>
-          <cell r="C95" t="str">
-            <v>#UsedGasVolume_H2</v>
-          </cell>
-          <cell r="D95" t="str">
-            <v>#LastUsedTime_MassFlowMeter</v>
-          </cell>
-        </row>
-        <row r="107">
-          <cell r="A107" t="str">
-            <v>#Balance</v>
-          </cell>
-          <cell r="B107" t="str">
-            <v>#LastUsedPurpose_Balance_BeforeFirstUse</v>
-          </cell>
-          <cell r="D107" t="str">
-            <v>#LastUsedTime_Balance</v>
-          </cell>
-        </row>
-        <row r="108">
-          <cell r="A108" t="str">
-            <v>#Balance</v>
-          </cell>
-          <cell r="B108" t="str">
-            <v>#DigitalObjectID_Balance</v>
-          </cell>
-        </row>
-        <row r="124">
-          <cell r="A124" t="str">
-            <v>#LiquidPhase</v>
-          </cell>
-          <cell r="C124" t="str">
-            <v>#Vessel_Energy</v>
-          </cell>
-          <cell r="E124" t="str">
-            <v>#Vessel_Space</v>
-          </cell>
-          <cell r="G124" t="str">
-            <v>#InitialMassFraction_Solvent_LiquidPhase</v>
-          </cell>
-        </row>
-        <row r="125">
-          <cell r="A125" t="str">
-            <v>#LiquidPhase</v>
-          </cell>
-          <cell r="E125" t="str">
-            <v>#Vessel_Structure</v>
-          </cell>
-          <cell r="G125" t="str">
-            <v>#InitialMassFraction_Water_LiquidPhase</v>
-          </cell>
-        </row>
-        <row r="126">
-          <cell r="A126" t="str">
-            <v>#LiquidPhase</v>
-          </cell>
-          <cell r="E126" t="str">
-            <v>#MaterialVolume_Reactor</v>
-          </cell>
-        </row>
-        <row r="127">
-          <cell r="A127" t="str">
-            <v>#LiquidPhase</v>
-          </cell>
-          <cell r="E127" t="str">
-            <v>#InitialVolume_LiquidPhase</v>
-          </cell>
-        </row>
-        <row r="137">
-          <cell r="A137" t="str">
-            <v>#SolidPhase</v>
-          </cell>
-          <cell r="C137" t="str">
-            <v>#Vessel_Energy</v>
-          </cell>
-          <cell r="E137" t="str">
-            <v>#Vessel_Space</v>
-          </cell>
-          <cell r="G137" t="str">
-            <v>#RDY_Energy</v>
-          </cell>
-        </row>
-        <row r="138">
-          <cell r="A138" t="str">
-            <v>#SolidPhase</v>
-          </cell>
-          <cell r="E138" t="str">
-            <v>#Vessel_Structure</v>
-          </cell>
-        </row>
-        <row r="139">
-          <cell r="A139" t="str">
-            <v>#SolidPhase</v>
-          </cell>
-          <cell r="E139" t="str">
-            <v>#MaterialVolume_Reactor</v>
-          </cell>
-        </row>
-        <row r="150">
-          <cell r="A150" t="str">
-            <v>#CatalystPhase</v>
-          </cell>
-          <cell r="C150" t="str">
-            <v>#Vessel_Energy</v>
-          </cell>
-          <cell r="E150" t="str">
-            <v>#Vessel_Space</v>
-          </cell>
-        </row>
-        <row r="151">
-          <cell r="A151" t="str">
-            <v>#CatalystPhase</v>
-          </cell>
-          <cell r="E151" t="str">
-            <v>#Vessel_Structure</v>
-          </cell>
-        </row>
-        <row r="152">
-          <cell r="A152" t="str">
-            <v>#CatalystPhase</v>
-          </cell>
-          <cell r="E152" t="str">
-            <v>#MaterialVolume_Reactor</v>
-          </cell>
-        </row>
-        <row r="163">
-          <cell r="A163" t="str">
-            <v>#GasPhase</v>
-          </cell>
-          <cell r="C163" t="str">
-            <v>#Vessel_Energy</v>
-          </cell>
-          <cell r="E163" t="str">
-            <v>#Vessel_Space</v>
-          </cell>
-        </row>
-        <row r="164">
-          <cell r="A164" t="str">
-            <v>#GasPhase</v>
-          </cell>
-          <cell r="E164" t="str">
-            <v>#Vessel_Structure</v>
-          </cell>
-        </row>
-        <row r="165">
-          <cell r="A165" t="str">
-            <v>#GasPhase</v>
-          </cell>
-          <cell r="E165" t="str">
-            <v>#MaterialVolume_Reactor</v>
-          </cell>
-        </row>
-        <row r="176">
-          <cell r="A176" t="str">
-            <v>#DispersedGasPhase</v>
-          </cell>
-          <cell r="C176" t="str">
-            <v>#Vessel_Energy</v>
-          </cell>
-          <cell r="E176" t="str">
-            <v>#Vessel_Space</v>
-          </cell>
-        </row>
-        <row r="177">
-          <cell r="A177" t="str">
-            <v>#DispersedGasPhase</v>
-          </cell>
-          <cell r="E177" t="str">
-            <v>#Vessel_Structure</v>
-          </cell>
-        </row>
-        <row r="178">
-          <cell r="A178" t="str">
-            <v>#DispersedGasPhase</v>
-          </cell>
-          <cell r="E178" t="str">
-            <v>#MaterialVolume_Reactor</v>
-          </cell>
-        </row>
-        <row r="189">
-          <cell r="A189" t="str">
-            <v>#CoolingFluidPhase</v>
-          </cell>
-          <cell r="C189" t="str">
-            <v>#Jacket_Energy</v>
-          </cell>
-          <cell r="E189" t="str">
-            <v>#Jacket_Space</v>
-          </cell>
-        </row>
-        <row r="190">
-          <cell r="A190" t="str">
-            <v>#CoolingFluidPhase</v>
-          </cell>
-          <cell r="C190" t="str">
-            <v>#SetFlowrateProfile_Jacket</v>
-          </cell>
-          <cell r="E190" t="str">
-            <v>#Jacket_Structure</v>
-          </cell>
-        </row>
-        <row r="191">
-          <cell r="A191" t="str">
-            <v>#CoolingFluidPhase</v>
-          </cell>
-          <cell r="E191" t="str">
-            <v>#CoolingFluidStream</v>
-          </cell>
-        </row>
-        <row r="202">
-          <cell r="A202" t="str">
-            <v>#HydrogenSpargerPhase</v>
-          </cell>
-          <cell r="C202" t="str">
-            <v>#Sparger_Energy</v>
-          </cell>
-          <cell r="E202" t="str">
-            <v>#Sparger_Space</v>
-          </cell>
-        </row>
-        <row r="203">
-          <cell r="A203" t="str">
-            <v>#HydrogenSpargerPhase</v>
-          </cell>
-          <cell r="E203" t="str">
-            <v>#Sparger_Structure</v>
-          </cell>
-        </row>
-        <row r="204">
-          <cell r="A204" t="str">
-            <v>#HydrogenSpargerPhase</v>
-          </cell>
-          <cell r="E204" t="str">
-            <v>#HydrogenStream</v>
-          </cell>
-        </row>
-        <row r="215">
-          <cell r="A215" t="str">
-            <v>#CleaningFluidPhase</v>
-          </cell>
-        </row>
-        <row r="231">
-          <cell r="A231" t="str">
-            <v>#H2</v>
-          </cell>
-          <cell r="C231" t="str">
-            <v>#GasPhase_Energy</v>
-          </cell>
-        </row>
-        <row r="232">
-          <cell r="A232" t="str">
-            <v>#H3</v>
-          </cell>
-          <cell r="C232" t="str">
-            <v>#DispersedGasPhase_Energy</v>
-          </cell>
-        </row>
-        <row r="233">
-          <cell r="A233" t="str">
-            <v>#H4</v>
-          </cell>
-          <cell r="C233" t="str">
-            <v>#HydrogenSpargerPhase_Energy</v>
-          </cell>
-        </row>
-        <row r="244">
-          <cell r="A244" t="str">
-            <v>#H2O</v>
-          </cell>
-          <cell r="C244" t="str">
-            <v>#LiquidPhase_Energy</v>
-          </cell>
-          <cell r="E244" t="str">
-            <v>#LiquidPhase_Space</v>
-          </cell>
-        </row>
-        <row r="245">
-          <cell r="E245" t="str">
-            <v>#InitialMassFraction_Water_LiquidPhase</v>
-          </cell>
-        </row>
-        <row r="257">
-          <cell r="A257" t="str">
-            <v>#Solvent</v>
-          </cell>
-          <cell r="C257" t="str">
-            <v>#LiquidPhase_Energy</v>
-          </cell>
-          <cell r="E257" t="str">
-            <v>#LiquidPhase_Space</v>
-          </cell>
-        </row>
-        <row r="258">
-          <cell r="E258" t="str">
-            <v>#InitialMassFraction_Solvent_LiquidPhase</v>
-          </cell>
-        </row>
-        <row r="270">
-          <cell r="A270" t="str">
-            <v>#RDY</v>
-          </cell>
-          <cell r="C270" t="str">
-            <v>#SolidPhase_Energy</v>
-          </cell>
-        </row>
-        <row r="271">
-          <cell r="A271" t="str">
-            <v>#RDY</v>
-          </cell>
-          <cell r="C271" t="str">
-            <v>#StartMass_RDY</v>
-          </cell>
-        </row>
-        <row r="272">
-          <cell r="A272" t="str">
-            <v>#RDY</v>
-          </cell>
-          <cell r="C272" t="str">
-            <v>#FinalMass_RDY</v>
-          </cell>
-        </row>
-        <row r="322">
-          <cell r="A322" t="str">
-            <v>#RDEt</v>
-          </cell>
-          <cell r="C322" t="str">
-            <v>#FinalMassRDEt</v>
-          </cell>
-        </row>
-        <row r="335">
-          <cell r="A335" t="str">
-            <v>#Dimer1</v>
-          </cell>
-          <cell r="C335" t="str">
-            <v>#FinalMass_Dimer</v>
-          </cell>
-        </row>
-        <row r="348">
-          <cell r="A348" t="str">
-            <v>#Dimer2</v>
-          </cell>
-          <cell r="C348" t="str">
-            <v>#FinalMass_Dimer</v>
-          </cell>
-        </row>
-        <row r="361">
-          <cell r="A361" t="str">
-            <v>#Pt</v>
-          </cell>
-          <cell r="C361" t="str">
-            <v>#CatalystPhase_Energy</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1076,9 +720,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED4507CF-D6FB-4A2B-A3A9-62CC9ECEF7FC}">
   <dimension ref="A1:G309"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -1101,19 +745,18 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="str" cm="1">
-        <f t="array" ref="A2:G11">[1]Context_Hydrogenation_New!A4:G13</f>
-        <v>#Reactor</v>
-      </c>
-      <c r="B2" t="str">
-        <v>#DigitalObjectID_Reactor</v>
-      </c>
-      <c r="C2" t="str">
-        <v>#TemperatureSensor_Energy</v>
-      </c>
-      <c r="D2" t="str">
-        <v>#LastUsedTime_Reactor</v>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1125,18 +768,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="str">
-        <v>#Reactor</v>
-      </c>
-      <c r="B3" t="str">
-        <v>#LastUsedPurpose_Reactor_BeforeFirstUse</v>
-      </c>
-      <c r="C3" t="str">
-        <v>#PressureSensor_Energy</v>
-      </c>
-      <c r="D3" t="str">
-        <v>#LastServicedTime_Reactor</v>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1148,18 +791,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="str">
-        <v>#Reactor</v>
-      </c>
-      <c r="B4" t="str">
-        <v>#OperatingMode_Reactor</v>
-      </c>
-      <c r="C4" t="str">
-        <v>#SetPressureProfile_Reactor</v>
-      </c>
-      <c r="D4" t="str">
-        <v>#ExperimentalProcedure</v>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1171,15 +814,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="str">
-        <v>#Reactor</v>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>7</v>
       </c>
       <c r="B5">
         <v>0</v>
       </c>
-      <c r="C5" t="str">
-        <v>#SetTemperatureProfile_Reactor</v>
+      <c r="C5" t="s">
+        <v>17</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -1194,7 +837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>0</v>
       </c>
@@ -1217,7 +860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>0</v>
       </c>
@@ -1240,7 +883,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>0</v>
       </c>
@@ -1263,7 +906,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>0</v>
       </c>
@@ -1286,7 +929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>0</v>
       </c>
@@ -1309,7 +952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>0</v>
       </c>
@@ -1332,19 +975,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" t="str" cm="1">
-        <f t="array" ref="A12:G22">[1]Context_Hydrogenation_New!A16:G26</f>
-        <v>#Vessel</v>
-      </c>
-      <c r="B12" t="str">
-        <v>#DigitalObjectID_Vessel</v>
-      </c>
-      <c r="C12" t="str">
-        <v>#Reactor_Energy</v>
-      </c>
-      <c r="D12" t="str">
-        <v>#LastUsedTime_Vessel</v>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" t="s">
+        <v>21</v>
       </c>
       <c r="E12">
         <v>0</v>
@@ -1356,18 +998,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" t="str">
-        <v>#Vessel</v>
-      </c>
-      <c r="B13" t="str">
-        <v>#LastUsedPurpose_Vessel_BeforeFirstUse</v>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" t="s">
+        <v>22</v>
       </c>
       <c r="C13">
         <v>0</v>
       </c>
-      <c r="D13" t="str">
-        <v>#Reactor_Time</v>
+      <c r="D13" t="s">
+        <v>23</v>
       </c>
       <c r="E13">
         <v>0</v>
@@ -1379,7 +1021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>0</v>
       </c>
@@ -1402,7 +1044,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>0</v>
       </c>
@@ -1425,7 +1067,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>0</v>
       </c>
@@ -1448,7 +1090,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>0</v>
       </c>
@@ -1471,7 +1113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>0</v>
       </c>
@@ -1494,7 +1136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>0</v>
       </c>
@@ -1517,7 +1159,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>0</v>
       </c>
@@ -1540,7 +1182,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>0</v>
       </c>
@@ -1563,7 +1205,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>0</v>
       </c>
@@ -1586,19 +1228,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" t="str" cm="1">
-        <f t="array" ref="A23:G33">[1]Context_Hydrogenation_New!A29:G39</f>
-        <v>#Stirrer</v>
-      </c>
-      <c r="B23" t="str">
-        <v>#DigitalObjectID_Stirrer</v>
-      </c>
-      <c r="C23" t="str">
-        <v>#Reactor_Energy</v>
-      </c>
-      <c r="D23" t="str">
-        <v>#LastUsedTime_Stirrer</v>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>24</v>
+      </c>
+      <c r="B23" t="s">
+        <v>25</v>
+      </c>
+      <c r="C23" t="s">
+        <v>20</v>
+      </c>
+      <c r="D23" t="s">
+        <v>26</v>
       </c>
       <c r="E23">
         <v>0</v>
@@ -1610,18 +1251,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" t="str">
-        <v>#Stirrer</v>
-      </c>
-      <c r="B24" t="str">
-        <v>#LastUsedPurpose_Stirrer_BeforeFirstUse</v>
-      </c>
-      <c r="C24" t="str">
-        <v>#SetRPMProfile_Reactor</v>
-      </c>
-      <c r="D24" t="str">
-        <v>#Reactor_Time</v>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>24</v>
+      </c>
+      <c r="B24" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" t="s">
+        <v>28</v>
+      </c>
+      <c r="D24" t="s">
+        <v>23</v>
       </c>
       <c r="E24">
         <v>0</v>
@@ -1633,7 +1274,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>0</v>
       </c>
@@ -1656,7 +1297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>0</v>
       </c>
@@ -1679,7 +1320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>0</v>
       </c>
@@ -1702,7 +1343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>0</v>
       </c>
@@ -1725,7 +1366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>0</v>
       </c>
@@ -1748,7 +1389,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>0</v>
       </c>
@@ -1771,7 +1412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>0</v>
       </c>
@@ -1794,7 +1435,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>0</v>
       </c>
@@ -1817,7 +1458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>0</v>
       </c>
@@ -1840,19 +1481,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" t="str" cm="1">
-        <f t="array" ref="A34:G44">[1]Context_Hydrogenation_New!A42:G52</f>
-        <v>#Sparger</v>
-      </c>
-      <c r="B34" t="str">
-        <v>#DigitalObjectID_Sparger</v>
-      </c>
-      <c r="C34" t="str">
-        <v>#Reactor_Energy</v>
-      </c>
-      <c r="D34" t="str">
-        <v>#LastUsedTime_Sparger</v>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>29</v>
+      </c>
+      <c r="B34" t="s">
+        <v>30</v>
+      </c>
+      <c r="C34" t="s">
+        <v>20</v>
+      </c>
+      <c r="D34" t="s">
+        <v>31</v>
       </c>
       <c r="E34">
         <v>0</v>
@@ -1864,18 +1504,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" t="str">
-        <v>#Sparger</v>
-      </c>
-      <c r="B35" t="str">
-        <v>#LastUsedPurpose_Sparger_BeforeFirstUse</v>
-      </c>
-      <c r="C35" t="str">
-        <v>#SetPressureProfile_Sparger</v>
-      </c>
-      <c r="D35" t="str">
-        <v>#Reactor_Time</v>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>29</v>
+      </c>
+      <c r="B35" t="s">
+        <v>32</v>
+      </c>
+      <c r="C35" t="s">
+        <v>33</v>
+      </c>
+      <c r="D35" t="s">
+        <v>23</v>
       </c>
       <c r="E35">
         <v>0</v>
@@ -1887,7 +1527,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>0</v>
       </c>
@@ -1910,7 +1550,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>0</v>
       </c>
@@ -1933,7 +1573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>0</v>
       </c>
@@ -1956,7 +1596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>0</v>
       </c>
@@ -1979,7 +1619,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>0</v>
       </c>
@@ -2002,7 +1642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>0</v>
       </c>
@@ -2025,7 +1665,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>0</v>
       </c>
@@ -2048,7 +1688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>0</v>
       </c>
@@ -2071,7 +1711,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>0</v>
       </c>
@@ -2094,19 +1734,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" t="str" cm="1">
-        <f t="array" ref="A45:G55">[1]Context_Hydrogenation_New!A55:G65</f>
-        <v>#Jacket</v>
-      </c>
-      <c r="B45" t="str">
-        <v>#DigitalObjectID_Jacket</v>
-      </c>
-      <c r="C45" t="str">
-        <v>#Reactor_Energy</v>
-      </c>
-      <c r="D45" t="str">
-        <v>#LastUsedTime_Jacket</v>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>34</v>
+      </c>
+      <c r="B45" t="s">
+        <v>35</v>
+      </c>
+      <c r="C45" t="s">
+        <v>20</v>
+      </c>
+      <c r="D45" t="s">
+        <v>36</v>
       </c>
       <c r="E45">
         <v>0</v>
@@ -2118,18 +1757,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" t="str">
-        <v>#Jacket</v>
-      </c>
-      <c r="B46" t="str">
-        <v>#LastUsedPurpose_Jacket_BeforeFirstUse</v>
-      </c>
-      <c r="C46" t="str">
-        <v>#SetFlowrateProfile_Jacket</v>
-      </c>
-      <c r="D46" t="str">
-        <v>#Reactor_Time</v>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>34</v>
+      </c>
+      <c r="B46" t="s">
+        <v>37</v>
+      </c>
+      <c r="C46" t="s">
+        <v>38</v>
+      </c>
+      <c r="D46" t="s">
+        <v>23</v>
       </c>
       <c r="E46">
         <v>0</v>
@@ -2141,7 +1780,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>0</v>
       </c>
@@ -2164,7 +1803,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>0</v>
       </c>
@@ -2187,7 +1826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>0</v>
       </c>
@@ -2210,7 +1849,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>0</v>
       </c>
@@ -2233,7 +1872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>0</v>
       </c>
@@ -2256,7 +1895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>0</v>
       </c>
@@ -2279,7 +1918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>0</v>
       </c>
@@ -2302,7 +1941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>0</v>
       </c>
@@ -2325,7 +1964,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>0</v>
       </c>
@@ -2348,19 +1987,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" t="str" cm="1">
-        <f t="array" ref="A56:G66">[1]Context_Hydrogenation_New!A68:G78</f>
-        <v>#TemperatureSensor</v>
-      </c>
-      <c r="B56" t="str">
-        <v>#LastUsedPurpose_TemperatureSensor_BeforeFirstUse</v>
-      </c>
-      <c r="C56" t="str">
-        <v>#Reactor_Energy</v>
-      </c>
-      <c r="D56" t="str">
-        <v>#Reactor_Time</v>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>39</v>
+      </c>
+      <c r="B56" t="s">
+        <v>40</v>
+      </c>
+      <c r="C56" t="s">
+        <v>20</v>
+      </c>
+      <c r="D56" t="s">
+        <v>23</v>
       </c>
       <c r="E56">
         <v>0</v>
@@ -2372,18 +2010,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" t="str">
-        <v>#TemperatureSensor</v>
-      </c>
-      <c r="B57" t="str">
-        <v>#DigitalObjectID_TemperatureSensor</v>
-      </c>
-      <c r="C57" t="str">
-        <v>#RecordedTemperature_Reactor</v>
-      </c>
-      <c r="D57" t="str">
-        <v>#LastUsedTime_TemperatureSensor</v>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>39</v>
+      </c>
+      <c r="B57" t="s">
+        <v>41</v>
+      </c>
+      <c r="C57" t="s">
+        <v>42</v>
+      </c>
+      <c r="D57" t="s">
+        <v>43</v>
       </c>
       <c r="E57">
         <v>0</v>
@@ -2395,7 +2033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>0</v>
       </c>
@@ -2418,7 +2056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>0</v>
       </c>
@@ -2441,7 +2079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>0</v>
       </c>
@@ -2464,7 +2102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>0</v>
       </c>
@@ -2487,7 +2125,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>0</v>
       </c>
@@ -2510,7 +2148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>0</v>
       </c>
@@ -2533,7 +2171,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>0</v>
       </c>
@@ -2556,7 +2194,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>0</v>
       </c>
@@ -2579,7 +2217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>0</v>
       </c>
@@ -2602,19 +2240,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A67" t="str" cm="1">
-        <f t="array" ref="A67:G77">[1]Context_Hydrogenation_New!A81:G91</f>
-        <v>#PressureSensor</v>
-      </c>
-      <c r="B67" t="str">
-        <v>#LastUsedPurpose_PressureSensor_BeforeFirstUse</v>
-      </c>
-      <c r="C67" t="str">
-        <v>#Reactor_Energy</v>
-      </c>
-      <c r="D67" t="str">
-        <v>#Reactor_Time</v>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>44</v>
+      </c>
+      <c r="B67" t="s">
+        <v>45</v>
+      </c>
+      <c r="C67" t="s">
+        <v>20</v>
+      </c>
+      <c r="D67" t="s">
+        <v>23</v>
       </c>
       <c r="E67">
         <v>0</v>
@@ -2626,18 +2263,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" t="str">
-        <v>#PressureSensor</v>
-      </c>
-      <c r="B68" t="str">
-        <v>#DigitalObjectID_PressureSensor</v>
-      </c>
-      <c r="C68" t="str">
-        <v>#RecordedPressure_Reactor</v>
-      </c>
-      <c r="D68" t="str">
-        <v>#LastUsedTime_PressureSensor</v>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>44</v>
+      </c>
+      <c r="B68" t="s">
+        <v>46</v>
+      </c>
+      <c r="C68" t="s">
+        <v>47</v>
+      </c>
+      <c r="D68" t="s">
+        <v>48</v>
       </c>
       <c r="E68">
         <v>0</v>
@@ -2649,7 +2286,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>0</v>
       </c>
@@ -2672,7 +2309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>0</v>
       </c>
@@ -2695,7 +2332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>0</v>
       </c>
@@ -2718,7 +2355,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>0</v>
       </c>
@@ -2741,7 +2378,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>0</v>
       </c>
@@ -2764,7 +2401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>0</v>
       </c>
@@ -2787,7 +2424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>0</v>
       </c>
@@ -2810,7 +2447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>0</v>
       </c>
@@ -2833,7 +2470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>0</v>
       </c>
@@ -2856,19 +2493,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A78" t="str" cm="1">
-        <f t="array" ref="A78:G88">[1]Context_Hydrogenation_New!A94:G104</f>
-        <v>#MassFlowMeter</v>
-      </c>
-      <c r="B78" t="str">
-        <v>#LastUsedPurpose_MassFlowMeter_BeforeFirstUse</v>
-      </c>
-      <c r="C78" t="str">
-        <v>#Reactor_Energy</v>
-      </c>
-      <c r="D78" t="str">
-        <v>#Reactor_Time</v>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>49</v>
+      </c>
+      <c r="B78" t="s">
+        <v>50</v>
+      </c>
+      <c r="C78" t="s">
+        <v>20</v>
+      </c>
+      <c r="D78" t="s">
+        <v>23</v>
       </c>
       <c r="E78">
         <v>0</v>
@@ -2880,18 +2516,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A79" t="str">
-        <v>#MassFlowMeter</v>
-      </c>
-      <c r="B79" t="str">
-        <v>#DigitalObjectID_MassFlowMeter</v>
-      </c>
-      <c r="C79" t="str">
-        <v>#UsedGasVolume_H2</v>
-      </c>
-      <c r="D79" t="str">
-        <v>#LastUsedTime_MassFlowMeter</v>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>49</v>
+      </c>
+      <c r="B79" t="s">
+        <v>51</v>
+      </c>
+      <c r="C79" t="s">
+        <v>52</v>
+      </c>
+      <c r="D79" t="s">
+        <v>53</v>
       </c>
       <c r="E79">
         <v>0</v>
@@ -2903,7 +2539,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>0</v>
       </c>
@@ -2926,7 +2562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>0</v>
       </c>
@@ -2949,7 +2585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>0</v>
       </c>
@@ -2972,7 +2608,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>0</v>
       </c>
@@ -2995,7 +2631,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>0</v>
       </c>
@@ -3018,7 +2654,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>0</v>
       </c>
@@ -3041,7 +2677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>0</v>
       </c>
@@ -3064,7 +2700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>0</v>
       </c>
@@ -3087,7 +2723,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>0</v>
       </c>
@@ -3110,19 +2746,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A89" t="str" cm="1">
-        <f t="array" ref="A89:G100">[1]Context_Hydrogenation_New!A107:G118</f>
-        <v>#Balance</v>
-      </c>
-      <c r="B89" t="str">
-        <v>#LastUsedPurpose_Balance_BeforeFirstUse</v>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>54</v>
+      </c>
+      <c r="B89" t="s">
+        <v>55</v>
       </c>
       <c r="C89">
         <v>0</v>
       </c>
-      <c r="D89" t="str">
-        <v>#LastUsedTime_Balance</v>
+      <c r="D89" t="s">
+        <v>56</v>
       </c>
       <c r="E89">
         <v>0</v>
@@ -3134,12 +2769,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A90" t="str">
-        <v>#Balance</v>
-      </c>
-      <c r="B90" t="str">
-        <v>#DigitalObjectID_Balance</v>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>54</v>
+      </c>
+      <c r="B90" t="s">
+        <v>57</v>
       </c>
       <c r="C90">
         <v>0</v>
@@ -3157,7 +2792,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>0</v>
       </c>
@@ -3180,7 +2815,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>0</v>
       </c>
@@ -3203,7 +2838,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>0</v>
       </c>
@@ -3226,7 +2861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>0</v>
       </c>
@@ -3249,7 +2884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>0</v>
       </c>
@@ -3272,7 +2907,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>0</v>
       </c>
@@ -3295,7 +2930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>0</v>
       </c>
@@ -3318,7 +2953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>0</v>
       </c>
@@ -3341,7 +2976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>0</v>
       </c>
@@ -3364,7 +2999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>0</v>
       </c>
@@ -3387,33 +3022,32 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A101" t="str" cm="1">
-        <f t="array" ref="A101:G111">[1]Context_Hydrogenation_New!A124:G134</f>
-        <v>#LiquidPhase</v>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
+        <v>58</v>
       </c>
       <c r="B101">
         <v>0</v>
       </c>
-      <c r="C101" t="str">
-        <v>#Vessel_Energy</v>
+      <c r="C101" t="s">
+        <v>59</v>
       </c>
       <c r="D101">
         <v>0</v>
       </c>
-      <c r="E101" t="str">
-        <v>#Vessel_Space</v>
+      <c r="E101" t="s">
+        <v>60</v>
       </c>
       <c r="F101">
         <v>0</v>
       </c>
-      <c r="G101" t="str">
-        <v>#InitialMassFraction_Solvent_LiquidPhase</v>
-      </c>
-    </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A102" t="str">
-        <v>#LiquidPhase</v>
+      <c r="G101" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A102" t="s">
+        <v>58</v>
       </c>
       <c r="B102">
         <v>0</v>
@@ -3424,19 +3058,19 @@
       <c r="D102">
         <v>0</v>
       </c>
-      <c r="E102" t="str">
-        <v>#Vessel_Structure</v>
+      <c r="E102" t="s">
+        <v>62</v>
       </c>
       <c r="F102">
         <v>0</v>
       </c>
-      <c r="G102" t="str">
-        <v>#InitialMassFraction_Water_LiquidPhase</v>
-      </c>
-    </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A103" t="str">
-        <v>#LiquidPhase</v>
+      <c r="G102" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>58</v>
       </c>
       <c r="B103">
         <v>0</v>
@@ -3447,8 +3081,8 @@
       <c r="D103">
         <v>0</v>
       </c>
-      <c r="E103" t="str">
-        <v>#MaterialVolume_Reactor</v>
+      <c r="E103" t="s">
+        <v>64</v>
       </c>
       <c r="F103">
         <v>0</v>
@@ -3457,9 +3091,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A104" t="str">
-        <v>#LiquidPhase</v>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A104" t="s">
+        <v>58</v>
       </c>
       <c r="B104">
         <v>0</v>
@@ -3470,8 +3104,8 @@
       <c r="D104">
         <v>0</v>
       </c>
-      <c r="E104" t="str">
-        <v>#InitialVolume_LiquidPhase</v>
+      <c r="E104" t="s">
+        <v>65</v>
       </c>
       <c r="F104">
         <v>0</v>
@@ -3480,7 +3114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>0</v>
       </c>
@@ -3503,7 +3137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>0</v>
       </c>
@@ -3526,7 +3160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>0</v>
       </c>
@@ -3549,7 +3183,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>0</v>
       </c>
@@ -3572,7 +3206,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>0</v>
       </c>
@@ -3595,7 +3229,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>0</v>
       </c>
@@ -3618,7 +3252,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>0</v>
       </c>
@@ -3641,33 +3275,32 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A112" t="str" cm="1">
-        <f t="array" ref="A112:G122">[1]Context_Hydrogenation_New!A137:G147</f>
-        <v>#SolidPhase</v>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A112" t="s">
+        <v>66</v>
       </c>
       <c r="B112">
         <v>0</v>
       </c>
-      <c r="C112" t="str">
-        <v>#Vessel_Energy</v>
+      <c r="C112" t="s">
+        <v>59</v>
       </c>
       <c r="D112">
         <v>0</v>
       </c>
-      <c r="E112" t="str">
-        <v>#Vessel_Space</v>
+      <c r="E112" t="s">
+        <v>60</v>
       </c>
       <c r="F112">
         <v>0</v>
       </c>
-      <c r="G112" t="str">
-        <v>#RDY_Energy</v>
-      </c>
-    </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A113" t="str">
-        <v>#SolidPhase</v>
+      <c r="G112" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A113" t="s">
+        <v>66</v>
       </c>
       <c r="B113">
         <v>0</v>
@@ -3678,8 +3311,8 @@
       <c r="D113">
         <v>0</v>
       </c>
-      <c r="E113" t="str">
-        <v>#Vessel_Structure</v>
+      <c r="E113" t="s">
+        <v>62</v>
       </c>
       <c r="F113">
         <v>0</v>
@@ -3688,9 +3321,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A114" t="str">
-        <v>#SolidPhase</v>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A114" t="s">
+        <v>66</v>
       </c>
       <c r="B114">
         <v>0</v>
@@ -3701,8 +3334,8 @@
       <c r="D114">
         <v>0</v>
       </c>
-      <c r="E114" t="str">
-        <v>#MaterialVolume_Reactor</v>
+      <c r="E114" t="s">
+        <v>64</v>
       </c>
       <c r="F114">
         <v>0</v>
@@ -3711,7 +3344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>0</v>
       </c>
@@ -3734,7 +3367,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>0</v>
       </c>
@@ -3757,7 +3390,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>0</v>
       </c>
@@ -3780,7 +3413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>0</v>
       </c>
@@ -3803,7 +3436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>0</v>
       </c>
@@ -3826,7 +3459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>0</v>
       </c>
@@ -3849,7 +3482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>0</v>
       </c>
@@ -3872,7 +3505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>0</v>
       </c>
@@ -3895,22 +3528,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A123" t="str" cm="1">
-        <f t="array" ref="A123:G133">[1]Context_Hydrogenation_New!A150:G160</f>
-        <v>#CatalystPhase</v>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A123" t="s">
+        <v>68</v>
       </c>
       <c r="B123">
         <v>0</v>
       </c>
-      <c r="C123" t="str">
-        <v>#Vessel_Energy</v>
+      <c r="C123" t="s">
+        <v>59</v>
       </c>
       <c r="D123">
         <v>0</v>
       </c>
-      <c r="E123" t="str">
-        <v>#Vessel_Space</v>
+      <c r="E123" t="s">
+        <v>60</v>
       </c>
       <c r="F123">
         <v>0</v>
@@ -3919,9 +3551,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A124" t="str">
-        <v>#CatalystPhase</v>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A124" t="s">
+        <v>68</v>
       </c>
       <c r="B124">
         <v>0</v>
@@ -3932,8 +3564,8 @@
       <c r="D124">
         <v>0</v>
       </c>
-      <c r="E124" t="str">
-        <v>#Vessel_Structure</v>
+      <c r="E124" t="s">
+        <v>62</v>
       </c>
       <c r="F124">
         <v>0</v>
@@ -3942,9 +3574,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A125" t="str">
-        <v>#CatalystPhase</v>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A125" t="s">
+        <v>68</v>
       </c>
       <c r="B125">
         <v>0</v>
@@ -3955,8 +3587,8 @@
       <c r="D125">
         <v>0</v>
       </c>
-      <c r="E125" t="str">
-        <v>#MaterialVolume_Reactor</v>
+      <c r="E125" t="s">
+        <v>64</v>
       </c>
       <c r="F125">
         <v>0</v>
@@ -3965,7 +3597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>0</v>
       </c>
@@ -3988,7 +3620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>0</v>
       </c>
@@ -4011,7 +3643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>0</v>
       </c>
@@ -4034,7 +3666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>0</v>
       </c>
@@ -4057,7 +3689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>0</v>
       </c>
@@ -4080,7 +3712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>0</v>
       </c>
@@ -4103,7 +3735,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>0</v>
       </c>
@@ -4126,7 +3758,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>0</v>
       </c>
@@ -4149,22 +3781,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A134" t="str" cm="1">
-        <f t="array" ref="A134:G144">[1]Context_Hydrogenation_New!A163:G173</f>
-        <v>#GasPhase</v>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A134" t="s">
+        <v>69</v>
       </c>
       <c r="B134">
         <v>0</v>
       </c>
-      <c r="C134" t="str">
-        <v>#Vessel_Energy</v>
+      <c r="C134" t="s">
+        <v>59</v>
       </c>
       <c r="D134">
         <v>0</v>
       </c>
-      <c r="E134" t="str">
-        <v>#Vessel_Space</v>
+      <c r="E134" t="s">
+        <v>60</v>
       </c>
       <c r="F134">
         <v>0</v>
@@ -4173,9 +3804,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A135" t="str">
-        <v>#GasPhase</v>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A135" t="s">
+        <v>69</v>
       </c>
       <c r="B135">
         <v>0</v>
@@ -4186,8 +3817,8 @@
       <c r="D135">
         <v>0</v>
       </c>
-      <c r="E135" t="str">
-        <v>#Vessel_Structure</v>
+      <c r="E135" t="s">
+        <v>62</v>
       </c>
       <c r="F135">
         <v>0</v>
@@ -4196,9 +3827,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A136" t="str">
-        <v>#GasPhase</v>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A136" t="s">
+        <v>69</v>
       </c>
       <c r="B136">
         <v>0</v>
@@ -4209,8 +3840,8 @@
       <c r="D136">
         <v>0</v>
       </c>
-      <c r="E136" t="str">
-        <v>#MaterialVolume_Reactor</v>
+      <c r="E136" t="s">
+        <v>64</v>
       </c>
       <c r="F136">
         <v>0</v>
@@ -4219,7 +3850,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>0</v>
       </c>
@@ -4242,7 +3873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>0</v>
       </c>
@@ -4265,7 +3896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>0</v>
       </c>
@@ -4288,7 +3919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>0</v>
       </c>
@@ -4311,7 +3942,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>0</v>
       </c>
@@ -4334,7 +3965,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>0</v>
       </c>
@@ -4357,7 +3988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>0</v>
       </c>
@@ -4380,7 +4011,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>0</v>
       </c>
@@ -4403,22 +4034,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A145" t="str" cm="1">
-        <f t="array" ref="A145:G155">[1]Context_Hydrogenation_New!A176:G186</f>
-        <v>#DispersedGasPhase</v>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A145" t="s">
+        <v>70</v>
       </c>
       <c r="B145">
         <v>0</v>
       </c>
-      <c r="C145" t="str">
-        <v>#Vessel_Energy</v>
+      <c r="C145" t="s">
+        <v>59</v>
       </c>
       <c r="D145">
         <v>0</v>
       </c>
-      <c r="E145" t="str">
-        <v>#Vessel_Space</v>
+      <c r="E145" t="s">
+        <v>60</v>
       </c>
       <c r="F145">
         <v>0</v>
@@ -4427,9 +4057,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A146" t="str">
-        <v>#DispersedGasPhase</v>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A146" t="s">
+        <v>70</v>
       </c>
       <c r="B146">
         <v>0</v>
@@ -4440,8 +4070,8 @@
       <c r="D146">
         <v>0</v>
       </c>
-      <c r="E146" t="str">
-        <v>#Vessel_Structure</v>
+      <c r="E146" t="s">
+        <v>62</v>
       </c>
       <c r="F146">
         <v>0</v>
@@ -4450,9 +4080,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A147" t="str">
-        <v>#DispersedGasPhase</v>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A147" t="s">
+        <v>70</v>
       </c>
       <c r="B147">
         <v>0</v>
@@ -4463,8 +4093,8 @@
       <c r="D147">
         <v>0</v>
       </c>
-      <c r="E147" t="str">
-        <v>#MaterialVolume_Reactor</v>
+      <c r="E147" t="s">
+        <v>64</v>
       </c>
       <c r="F147">
         <v>0</v>
@@ -4473,7 +4103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>0</v>
       </c>
@@ -4496,7 +4126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>0</v>
       </c>
@@ -4519,7 +4149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>0</v>
       </c>
@@ -4542,7 +4172,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>0</v>
       </c>
@@ -4565,7 +4195,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>0</v>
       </c>
@@ -4588,7 +4218,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>0</v>
       </c>
@@ -4611,7 +4241,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>0</v>
       </c>
@@ -4634,7 +4264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>0</v>
       </c>
@@ -4657,22 +4287,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A156" t="str" cm="1">
-        <f t="array" ref="A156:G166">[1]Context_Hydrogenation_New!A189:G199</f>
-        <v>#CoolingFluidPhase</v>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A156" t="s">
+        <v>71</v>
       </c>
       <c r="B156">
         <v>0</v>
       </c>
-      <c r="C156" t="str">
-        <v>#Jacket_Energy</v>
+      <c r="C156" t="s">
+        <v>72</v>
       </c>
       <c r="D156">
         <v>0</v>
       </c>
-      <c r="E156" t="str">
-        <v>#Jacket_Space</v>
+      <c r="E156" t="s">
+        <v>73</v>
       </c>
       <c r="F156">
         <v>0</v>
@@ -4681,21 +4310,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A157" t="str">
-        <v>#CoolingFluidPhase</v>
+    <row r="157" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A157" t="s">
+        <v>71</v>
       </c>
       <c r="B157">
         <v>0</v>
       </c>
-      <c r="C157" t="str">
-        <v>#SetFlowrateProfile_Jacket</v>
+      <c r="C157">
+        <v>0</v>
       </c>
       <c r="D157">
         <v>0</v>
       </c>
-      <c r="E157" t="str">
-        <v>#Jacket_Structure</v>
+      <c r="E157" t="s">
+        <v>74</v>
       </c>
       <c r="F157">
         <v>0</v>
@@ -4704,9 +4333,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A158" t="str">
-        <v>#CoolingFluidPhase</v>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A158" t="s">
+        <v>71</v>
       </c>
       <c r="B158">
         <v>0</v>
@@ -4717,8 +4346,8 @@
       <c r="D158">
         <v>0</v>
       </c>
-      <c r="E158" t="str">
-        <v>#CoolingFluidStream</v>
+      <c r="E158" t="s">
+        <v>75</v>
       </c>
       <c r="F158">
         <v>0</v>
@@ -4727,7 +4356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>0</v>
       </c>
@@ -4750,7 +4379,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>0</v>
       </c>
@@ -4773,7 +4402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>0</v>
       </c>
@@ -4796,7 +4425,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>0</v>
       </c>
@@ -4819,7 +4448,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>0</v>
       </c>
@@ -4842,7 +4471,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>0</v>
       </c>
@@ -4865,7 +4494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>0</v>
       </c>
@@ -4888,7 +4517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>0</v>
       </c>
@@ -4911,22 +4540,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A167" t="str" cm="1">
-        <f t="array" ref="A167:G177">[1]Context_Hydrogenation_New!A202:G212</f>
-        <v>#HydrogenSpargerPhase</v>
+    <row r="167" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A167" t="s">
+        <v>76</v>
       </c>
       <c r="B167">
         <v>0</v>
       </c>
-      <c r="C167" t="str">
-        <v>#Sparger_Energy</v>
+      <c r="C167" t="s">
+        <v>77</v>
       </c>
       <c r="D167">
         <v>0</v>
       </c>
-      <c r="E167" t="str">
-        <v>#Sparger_Space</v>
+      <c r="E167" t="s">
+        <v>78</v>
       </c>
       <c r="F167">
         <v>0</v>
@@ -4935,9 +4563,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A168" t="str">
-        <v>#HydrogenSpargerPhase</v>
+    <row r="168" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A168" t="s">
+        <v>76</v>
       </c>
       <c r="B168">
         <v>0</v>
@@ -4948,8 +4576,8 @@
       <c r="D168">
         <v>0</v>
       </c>
-      <c r="E168" t="str">
-        <v>#Sparger_Structure</v>
+      <c r="E168" t="s">
+        <v>79</v>
       </c>
       <c r="F168">
         <v>0</v>
@@ -4958,9 +4586,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A169" t="str">
-        <v>#HydrogenSpargerPhase</v>
+    <row r="169" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A169" t="s">
+        <v>76</v>
       </c>
       <c r="B169">
         <v>0</v>
@@ -4971,8 +4599,8 @@
       <c r="D169">
         <v>0</v>
       </c>
-      <c r="E169" t="str">
-        <v>#HydrogenStream</v>
+      <c r="E169" t="s">
+        <v>80</v>
       </c>
       <c r="F169">
         <v>0</v>
@@ -4981,7 +4609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>0</v>
       </c>
@@ -5004,7 +4632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>0</v>
       </c>
@@ -5027,7 +4655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>0</v>
       </c>
@@ -5050,7 +4678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>0</v>
       </c>
@@ -5073,7 +4701,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>0</v>
       </c>
@@ -5096,7 +4724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>0</v>
       </c>
@@ -5119,7 +4747,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>0</v>
       </c>
@@ -5142,7 +4770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>0</v>
       </c>
@@ -5165,10 +4793,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A178" t="str" cm="1">
-        <f t="array" ref="A178:G188">[1]Context_Hydrogenation_New!A215:G225</f>
-        <v>#CleaningFluidPhase</v>
+    <row r="178" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A178" t="s">
+        <v>81</v>
       </c>
       <c r="B178">
         <v>0</v>
@@ -5189,7 +4816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>0</v>
       </c>
@@ -5212,7 +4839,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>0</v>
       </c>
@@ -5235,7 +4862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>0</v>
       </c>
@@ -5258,7 +4885,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>0</v>
       </c>
@@ -5281,7 +4908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>0</v>
       </c>
@@ -5304,7 +4931,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>0</v>
       </c>
@@ -5327,7 +4954,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>0</v>
       </c>
@@ -5350,7 +4977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>0</v>
       </c>
@@ -5373,7 +5000,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A187">
         <v>0</v>
       </c>
@@ -5396,7 +5023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A188">
         <v>0</v>
       </c>
@@ -5419,16 +5046,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A189" t="str" cm="1">
-        <f t="array" ref="A189:G199">[1]Context_Hydrogenation_New!A231:G241</f>
-        <v>#H2</v>
+    <row r="189" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A189" t="s">
+        <v>82</v>
       </c>
       <c r="B189">
         <v>0</v>
       </c>
-      <c r="C189" t="str">
-        <v>#GasPhase_Energy</v>
+      <c r="C189" t="s">
+        <v>83</v>
       </c>
       <c r="D189">
         <v>0</v>
@@ -5443,15 +5069,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A190" t="str">
-        <v>#H3</v>
+    <row r="190" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A190" t="s">
+        <v>84</v>
       </c>
       <c r="B190">
         <v>0</v>
       </c>
-      <c r="C190" t="str">
-        <v>#DispersedGasPhase_Energy</v>
+      <c r="C190" t="s">
+        <v>85</v>
       </c>
       <c r="D190">
         <v>0</v>
@@ -5466,15 +5092,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A191" t="str">
-        <v>#H4</v>
+    <row r="191" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A191" t="s">
+        <v>86</v>
       </c>
       <c r="B191">
         <v>0</v>
       </c>
-      <c r="C191" t="str">
-        <v>#HydrogenSpargerPhase_Energy</v>
+      <c r="C191" t="s">
+        <v>87</v>
       </c>
       <c r="D191">
         <v>0</v>
@@ -5489,7 +5115,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>0</v>
       </c>
@@ -5512,7 +5138,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>0</v>
       </c>
@@ -5535,7 +5161,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>0</v>
       </c>
@@ -5558,7 +5184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>0</v>
       </c>
@@ -5581,7 +5207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>0</v>
       </c>
@@ -5604,7 +5230,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A197">
         <v>0</v>
       </c>
@@ -5627,7 +5253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>0</v>
       </c>
@@ -5650,7 +5276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A199">
         <v>0</v>
       </c>
@@ -5673,22 +5299,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A200" t="str" cm="1">
-        <f t="array" ref="A200:G210">[1]Context_Hydrogenation_New!A244:G254</f>
-        <v>#H2O</v>
+    <row r="200" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A200" t="s">
+        <v>88</v>
       </c>
       <c r="B200">
         <v>0</v>
       </c>
-      <c r="C200" t="str">
-        <v>#LiquidPhase_Energy</v>
+      <c r="C200" t="s">
+        <v>89</v>
       </c>
       <c r="D200">
         <v>0</v>
       </c>
-      <c r="E200" t="str">
-        <v>#LiquidPhase_Space</v>
+      <c r="E200" t="s">
+        <v>90</v>
       </c>
       <c r="F200">
         <v>0</v>
@@ -5697,7 +5322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>0</v>
       </c>
@@ -5710,8 +5335,8 @@
       <c r="D201">
         <v>0</v>
       </c>
-      <c r="E201" t="str">
-        <v>#InitialMassFraction_Water_LiquidPhase</v>
+      <c r="E201">
+        <v>0</v>
       </c>
       <c r="F201">
         <v>0</v>
@@ -5720,7 +5345,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>0</v>
       </c>
@@ -5743,7 +5368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A203">
         <v>0</v>
       </c>
@@ -5766,7 +5391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>0</v>
       </c>
@@ -5789,7 +5414,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>0</v>
       </c>
@@ -5812,7 +5437,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A206">
         <v>0</v>
       </c>
@@ -5835,7 +5460,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>0</v>
       </c>
@@ -5858,7 +5483,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>0</v>
       </c>
@@ -5881,7 +5506,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A209">
         <v>0</v>
       </c>
@@ -5904,7 +5529,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A210">
         <v>0</v>
       </c>
@@ -5927,22 +5552,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A211" t="str" cm="1">
-        <f t="array" ref="A211:G221">[1]Context_Hydrogenation_New!A257:G267</f>
-        <v>#Solvent</v>
+    <row r="211" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A211" t="s">
+        <v>91</v>
       </c>
       <c r="B211">
         <v>0</v>
       </c>
-      <c r="C211" t="str">
-        <v>#LiquidPhase_Energy</v>
+      <c r="C211" t="s">
+        <v>89</v>
       </c>
       <c r="D211">
         <v>0</v>
       </c>
-      <c r="E211" t="str">
-        <v>#LiquidPhase_Space</v>
+      <c r="E211" t="s">
+        <v>90</v>
       </c>
       <c r="F211">
         <v>0</v>
@@ -5951,7 +5575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A212">
         <v>0</v>
       </c>
@@ -5964,8 +5588,8 @@
       <c r="D212">
         <v>0</v>
       </c>
-      <c r="E212" t="str">
-        <v>#InitialMassFraction_Solvent_LiquidPhase</v>
+      <c r="E212">
+        <v>0</v>
       </c>
       <c r="F212">
         <v>0</v>
@@ -5974,7 +5598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A213">
         <v>0</v>
       </c>
@@ -5997,7 +5621,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A214">
         <v>0</v>
       </c>
@@ -6020,7 +5644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A215">
         <v>0</v>
       </c>
@@ -6043,7 +5667,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A216">
         <v>0</v>
       </c>
@@ -6066,7 +5690,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A217">
         <v>0</v>
       </c>
@@ -6089,7 +5713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A218">
         <v>0</v>
       </c>
@@ -6112,7 +5736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A219">
         <v>0</v>
       </c>
@@ -6135,7 +5759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A220">
         <v>0</v>
       </c>
@@ -6158,7 +5782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A221">
         <v>0</v>
       </c>
@@ -6181,16 +5805,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A222" t="str" cm="1">
-        <f t="array" ref="A222:G232">[1]Context_Hydrogenation_New!A270:G280</f>
-        <v>#RDY</v>
+    <row r="222" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A222" t="s">
+        <v>92</v>
       </c>
       <c r="B222">
         <v>0</v>
       </c>
-      <c r="C222" t="str">
-        <v>#SolidPhase_Energy</v>
+      <c r="C222" t="s">
+        <v>93</v>
       </c>
       <c r="D222">
         <v>0</v>
@@ -6205,15 +5828,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A223" t="str">
-        <v>#RDY</v>
+    <row r="223" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A223" t="s">
+        <v>92</v>
       </c>
       <c r="B223">
         <v>0</v>
       </c>
-      <c r="C223" t="str">
-        <v>#StartMass_RDY</v>
+      <c r="C223" t="s">
+        <v>94</v>
       </c>
       <c r="D223">
         <v>0</v>
@@ -6228,15 +5851,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A224" t="str">
-        <v>#RDY</v>
+    <row r="224" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A224" t="s">
+        <v>92</v>
       </c>
       <c r="B224">
         <v>0</v>
       </c>
-      <c r="C224" t="str">
-        <v>#FinalMass_RDY</v>
+      <c r="C224" t="s">
+        <v>95</v>
       </c>
       <c r="D224">
         <v>0</v>
@@ -6251,7 +5874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A225">
         <v>0</v>
       </c>
@@ -6274,7 +5897,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A226">
         <v>0</v>
       </c>
@@ -6297,7 +5920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A227">
         <v>0</v>
       </c>
@@ -6320,7 +5943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A228">
         <v>0</v>
       </c>
@@ -6343,7 +5966,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A229">
         <v>0</v>
       </c>
@@ -6366,7 +5989,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="230" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A230">
         <v>0</v>
       </c>
@@ -6389,7 +6012,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="231" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A231">
         <v>0</v>
       </c>
@@ -6412,7 +6035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="232" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A232">
         <v>0</v>
       </c>
@@ -6435,9 +6058,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="233" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A233" cm="1">
-        <f t="array" ref="A233:G243">[1]Context_Hydrogenation_New!A283:G293</f>
+    <row r="233" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A233">
         <v>0</v>
       </c>
       <c r="B233">
@@ -6459,7 +6081,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="234" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A234">
         <v>0</v>
       </c>
@@ -6482,7 +6104,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="235" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A235">
         <v>0</v>
       </c>
@@ -6505,7 +6127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="236" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A236">
         <v>0</v>
       </c>
@@ -6528,7 +6150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="237" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A237">
         <v>0</v>
       </c>
@@ -6551,7 +6173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="238" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A238">
         <v>0</v>
       </c>
@@ -6574,7 +6196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="239" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A239">
         <v>0</v>
       </c>
@@ -6597,7 +6219,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="240" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A240">
         <v>0</v>
       </c>
@@ -6620,7 +6242,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="241" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A241">
         <v>0</v>
       </c>
@@ -6643,7 +6265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="242" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A242">
         <v>0</v>
       </c>
@@ -6666,7 +6288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="243" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A243">
         <v>0</v>
       </c>
@@ -6689,9 +6311,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="244" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A244" cm="1">
-        <f t="array" ref="A244:G254">[1]Context_Hydrogenation_New!A296:G306</f>
+    <row r="244" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A244">
         <v>0</v>
       </c>
       <c r="B244">
@@ -6713,7 +6334,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="245" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A245">
         <v>0</v>
       </c>
@@ -6736,7 +6357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="246" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A246">
         <v>0</v>
       </c>
@@ -6759,7 +6380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="247" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A247">
         <v>0</v>
       </c>
@@ -6782,7 +6403,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A248">
         <v>0</v>
       </c>
@@ -6805,7 +6426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="249" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A249">
         <v>0</v>
       </c>
@@ -6828,7 +6449,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="250" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A250">
         <v>0</v>
       </c>
@@ -6851,7 +6472,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="251" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A251">
         <v>0</v>
       </c>
@@ -6874,7 +6495,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="252" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A252">
         <v>0</v>
       </c>
@@ -6897,7 +6518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="253" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A253">
         <v>0</v>
       </c>
@@ -6920,7 +6541,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="254" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A254">
         <v>0</v>
       </c>
@@ -6943,9 +6564,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="255" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A255" cm="1">
-        <f t="array" ref="A255:G265">[1]Context_Hydrogenation_New!A309:G319</f>
+    <row r="255" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A255">
         <v>0</v>
       </c>
       <c r="B255">
@@ -6967,7 +6587,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="256" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A256">
         <v>0</v>
       </c>
@@ -6990,7 +6610,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="257" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A257">
         <v>0</v>
       </c>
@@ -7013,7 +6633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="258" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A258">
         <v>0</v>
       </c>
@@ -7036,7 +6656,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="259" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A259">
         <v>0</v>
       </c>
@@ -7059,7 +6679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="260" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A260">
         <v>0</v>
       </c>
@@ -7082,7 +6702,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="261" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A261">
         <v>0</v>
       </c>
@@ -7105,7 +6725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="262" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A262">
         <v>0</v>
       </c>
@@ -7128,7 +6748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="263" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A263">
         <v>0</v>
       </c>
@@ -7151,7 +6771,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="264" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A264">
         <v>0</v>
       </c>
@@ -7174,7 +6794,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="265" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A265">
         <v>0</v>
       </c>
@@ -7197,16 +6817,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="266" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A266" t="str" cm="1">
-        <f t="array" ref="A266:G276">[1]Context_Hydrogenation_New!A322:G332</f>
-        <v>#RDEt</v>
+    <row r="266" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A266" t="s">
+        <v>96</v>
       </c>
       <c r="B266">
         <v>0</v>
       </c>
-      <c r="C266" t="str">
-        <v>#FinalMassRDEt</v>
+      <c r="C266" t="s">
+        <v>97</v>
       </c>
       <c r="D266">
         <v>0</v>
@@ -7221,7 +6840,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="267" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A267">
         <v>0</v>
       </c>
@@ -7244,7 +6863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="268" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A268">
         <v>0</v>
       </c>
@@ -7267,7 +6886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="269" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A269">
         <v>0</v>
       </c>
@@ -7290,7 +6909,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="270" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A270">
         <v>0</v>
       </c>
@@ -7313,7 +6932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="271" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A271">
         <v>0</v>
       </c>
@@ -7336,7 +6955,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="272" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A272">
         <v>0</v>
       </c>
@@ -7359,7 +6978,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="273" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A273">
         <v>0</v>
       </c>
@@ -7382,7 +7001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="274" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A274">
         <v>0</v>
       </c>
@@ -7405,7 +7024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="275" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A275">
         <v>0</v>
       </c>
@@ -7428,7 +7047,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="276" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A276">
         <v>0</v>
       </c>
@@ -7451,16 +7070,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="277" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A277" t="str" cm="1">
-        <f t="array" ref="A277:G287">[1]Context_Hydrogenation_New!A335:G345</f>
-        <v>#Dimer1</v>
+    <row r="277" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A277" t="s">
+        <v>98</v>
       </c>
       <c r="B277">
         <v>0</v>
       </c>
-      <c r="C277" t="str">
-        <v>#FinalMass_Dimer</v>
+      <c r="C277" t="s">
+        <v>99</v>
       </c>
       <c r="D277">
         <v>0</v>
@@ -7475,7 +7093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="278" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A278">
         <v>0</v>
       </c>
@@ -7498,7 +7116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="279" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A279">
         <v>0</v>
       </c>
@@ -7521,7 +7139,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="280" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A280">
         <v>0</v>
       </c>
@@ -7544,7 +7162,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="281" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A281">
         <v>0</v>
       </c>
@@ -7567,7 +7185,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="282" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A282">
         <v>0</v>
       </c>
@@ -7590,7 +7208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="283" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A283">
         <v>0</v>
       </c>
@@ -7613,7 +7231,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="284" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A284">
         <v>0</v>
       </c>
@@ -7636,7 +7254,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="285" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A285">
         <v>0</v>
       </c>
@@ -7659,7 +7277,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="286" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A286">
         <v>0</v>
       </c>
@@ -7682,7 +7300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="287" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A287">
         <v>0</v>
       </c>
@@ -7705,16 +7323,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="288" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A288" t="str" cm="1">
-        <f t="array" ref="A288:G298">[1]Context_Hydrogenation_New!A348:G358</f>
-        <v>#Dimer2</v>
+    <row r="288" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A288" t="s">
+        <v>100</v>
       </c>
       <c r="B288">
         <v>0</v>
       </c>
-      <c r="C288" t="str">
-        <v>#FinalMass_Dimer</v>
+      <c r="C288" t="s">
+        <v>99</v>
       </c>
       <c r="D288">
         <v>0</v>
@@ -7729,7 +7346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="289" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A289">
         <v>0</v>
       </c>
@@ -7752,7 +7369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="290" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A290">
         <v>0</v>
       </c>
@@ -7775,7 +7392,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="291" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A291">
         <v>0</v>
       </c>
@@ -7798,7 +7415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="292" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A292">
         <v>0</v>
       </c>
@@ -7821,7 +7438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="293" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A293">
         <v>0</v>
       </c>
@@ -7844,7 +7461,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="294" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A294">
         <v>0</v>
       </c>
@@ -7867,7 +7484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="295" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A295">
         <v>0</v>
       </c>
@@ -7890,7 +7507,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="296" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A296">
         <v>0</v>
       </c>
@@ -7913,7 +7530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="297" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A297">
         <v>0</v>
       </c>
@@ -7936,7 +7553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="298" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A298">
         <v>0</v>
       </c>
@@ -7959,16 +7576,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="299" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A299" t="str" cm="1">
-        <f t="array" ref="A299:G309">[1]Context_Hydrogenation_New!A361:G371</f>
-        <v>#Pt</v>
+    <row r="299" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A299" t="s">
+        <v>101</v>
       </c>
       <c r="B299">
         <v>0</v>
       </c>
-      <c r="C299" t="str">
-        <v>#CatalystPhase_Energy</v>
+      <c r="C299" t="s">
+        <v>102</v>
       </c>
       <c r="D299">
         <v>0</v>
@@ -7983,7 +7599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="300" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A300">
         <v>0</v>
       </c>
@@ -8006,7 +7622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="301" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A301">
         <v>0</v>
       </c>
@@ -8029,7 +7645,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="302" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A302">
         <v>0</v>
       </c>
@@ -8052,7 +7668,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="303" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A303">
         <v>0</v>
       </c>
@@ -8075,7 +7691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="304" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A304">
         <v>0</v>
       </c>
@@ -8098,7 +7714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="305" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A305">
         <v>0</v>
       </c>
@@ -8121,7 +7737,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="306" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A306">
         <v>0</v>
       </c>
@@ -8144,7 +7760,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="307" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A307">
         <v>0</v>
       </c>
@@ -8167,7 +7783,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="308" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A308">
         <v>0</v>
       </c>
@@ -8190,7 +7806,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="309" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A309">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Aufteilen der Skriptanweisungen in separate Textdatei
</commit_message>
<xml_diff>
--- a/context_connections.xlsx
+++ b/context_connections.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofcambridgecloud-my.sharepoint.com/personal/lf576_cam_ac_uk/Documents/04_Coding/hydrogenation/current_versions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="8_{C5C5D99A-F90E-4DDA-B551-364ECC0B9EB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0208EC85-E801-4E12-8B40-E93C03BCFA46}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="8_{C5C5D99A-F90E-4DDA-B551-364ECC0B9EB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E6A8B7AD-1E7C-47F1-8A13-20457BB0667C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2AABB6A2-CE1B-404B-9F86-D510FD910096}"/>
+    <workbookView minimized="1" xWindow="-37605" yWindow="2400" windowWidth="28590" windowHeight="15240" xr2:uid="{2AABB6A2-CE1B-404B-9F86-D510FD910096}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -408,6 +408,9 @@
           <cell r="B107" t="str">
             <v>#LastUsedPurpose_Balance_BeforeFirstUse</v>
           </cell>
+          <cell r="C107" t="str">
+            <v>#StartMassRDY</v>
+          </cell>
           <cell r="D107" t="str">
             <v>#LastUsedTime_Balance</v>
           </cell>
@@ -419,6 +422,19 @@
           <cell r="B108" t="str">
             <v>#DigitalObjectID_Balance</v>
           </cell>
+          <cell r="C108" t="str">
+            <v>#FinalMass_RDY</v>
+          </cell>
+        </row>
+        <row r="109">
+          <cell r="C109" t="str">
+            <v>#FinalMass_RDEt</v>
+          </cell>
+        </row>
+        <row r="110">
+          <cell r="C110" t="str">
+            <v>#FinalMass_Dimer</v>
+          </cell>
         </row>
         <row r="124">
           <cell r="A124" t="str">
@@ -452,6 +468,9 @@
           <cell r="E126" t="str">
             <v>#MaterialVolume_Reactor</v>
           </cell>
+          <cell r="G126" t="str">
+            <v>#Reaction1</v>
+          </cell>
         </row>
         <row r="127">
           <cell r="A127" t="str">
@@ -460,6 +479,14 @@
           <cell r="E127" t="str">
             <v>#InitialVolume_LiquidPhase</v>
           </cell>
+          <cell r="G127" t="str">
+            <v>#Reaction2</v>
+          </cell>
+        </row>
+        <row r="128">
+          <cell r="G128" t="str">
+            <v>#Reaction3</v>
+          </cell>
         </row>
         <row r="137">
           <cell r="A137" t="str">
@@ -482,6 +509,9 @@
           <cell r="E138" t="str">
             <v>#Vessel_Structure</v>
           </cell>
+          <cell r="G138" t="str">
+            <v>#Reaction1</v>
+          </cell>
         </row>
         <row r="139">
           <cell r="A139" t="str">
@@ -501,6 +531,9 @@
           <cell r="E150" t="str">
             <v>#Vessel_Space</v>
           </cell>
+          <cell r="G150" t="str">
+            <v>#Reaction1</v>
+          </cell>
         </row>
         <row r="151">
           <cell r="A151" t="str">
@@ -509,6 +542,9 @@
           <cell r="E151" t="str">
             <v>#Vessel_Structure</v>
           </cell>
+          <cell r="G151" t="str">
+            <v>#Reaction2</v>
+          </cell>
         </row>
         <row r="152">
           <cell r="A152" t="str">
@@ -517,6 +553,9 @@
           <cell r="E152" t="str">
             <v>#MaterialVolume_Reactor</v>
           </cell>
+          <cell r="G152" t="str">
+            <v>#Reaction3</v>
+          </cell>
         </row>
         <row r="163">
           <cell r="A163" t="str">
@@ -554,6 +593,9 @@
           </cell>
           <cell r="E176" t="str">
             <v>#Vessel_Space</v>
+          </cell>
+          <cell r="G176" t="str">
+            <v>#Reaction1</v>
           </cell>
         </row>
         <row r="177">
@@ -1059,9 +1101,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED4507CF-D6FB-4A2B-A3A9-62CC9ECEF7FC}">
   <dimension ref="A1:G309"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -1084,7 +1126,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="str" cm="1">
         <f t="array" ref="A2:G11">[1]Context_Input!A4:G13</f>
         <v>#Reactor</v>
@@ -1108,7 +1150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
         <v>#Reactor</v>
       </c>
@@ -1131,7 +1173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
         <v>#Reactor</v>
       </c>
@@ -1154,7 +1196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
         <v>#Reactor</v>
       </c>
@@ -1177,7 +1219,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>0</v>
       </c>
@@ -1200,7 +1242,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>0</v>
       </c>
@@ -1223,7 +1265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>0</v>
       </c>
@@ -1246,7 +1288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>0</v>
       </c>
@@ -1269,7 +1311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>0</v>
       </c>
@@ -1292,7 +1334,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>0</v>
       </c>
@@ -1315,7 +1357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="str" cm="1">
         <f t="array" ref="A12:G22">[1]Context_Input!A16:G26</f>
         <v>#Vessel</v>
@@ -1339,7 +1381,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="str">
         <v>#Vessel</v>
       </c>
@@ -1362,7 +1404,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>0</v>
       </c>
@@ -1385,7 +1427,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>0</v>
       </c>
@@ -1408,7 +1450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>0</v>
       </c>
@@ -1431,7 +1473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>0</v>
       </c>
@@ -1454,7 +1496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>0</v>
       </c>
@@ -1477,7 +1519,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>0</v>
       </c>
@@ -1500,7 +1542,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>0</v>
       </c>
@@ -1523,7 +1565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>0</v>
       </c>
@@ -1546,7 +1588,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>0</v>
       </c>
@@ -1569,7 +1611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="str" cm="1">
         <f t="array" ref="A23:G33">[1]Context_Input!A29:G39</f>
         <v>#Stirrer</v>
@@ -1593,7 +1635,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="str">
         <v>#Stirrer</v>
       </c>
@@ -1616,7 +1658,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>0</v>
       </c>
@@ -1639,7 +1681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>0</v>
       </c>
@@ -1662,7 +1704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>0</v>
       </c>
@@ -1685,7 +1727,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>0</v>
       </c>
@@ -1708,7 +1750,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>0</v>
       </c>
@@ -1731,7 +1773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>0</v>
       </c>
@@ -1754,7 +1796,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>0</v>
       </c>
@@ -1777,7 +1819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>0</v>
       </c>
@@ -1800,7 +1842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>0</v>
       </c>
@@ -1823,7 +1865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="str" cm="1">
         <f t="array" ref="A34:G44">[1]Context_Input!A42:G52</f>
         <v>#Sparger</v>
@@ -1847,7 +1889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="str">
         <v>#Sparger</v>
       </c>
@@ -1870,7 +1912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>0</v>
       </c>
@@ -1893,7 +1935,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>0</v>
       </c>
@@ -1916,7 +1958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>0</v>
       </c>
@@ -1939,7 +1981,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>0</v>
       </c>
@@ -1962,7 +2004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>0</v>
       </c>
@@ -1985,7 +2027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>0</v>
       </c>
@@ -2008,7 +2050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>0</v>
       </c>
@@ -2031,7 +2073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>0</v>
       </c>
@@ -2054,7 +2096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>0</v>
       </c>
@@ -2077,7 +2119,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="str" cm="1">
         <f t="array" ref="A45:G55">[1]Context_Input!A55:G65</f>
         <v>#Jacket</v>
@@ -2101,7 +2143,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="str">
         <v>#Jacket</v>
       </c>
@@ -2124,7 +2166,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>0</v>
       </c>
@@ -2147,7 +2189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>0</v>
       </c>
@@ -2170,7 +2212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>0</v>
       </c>
@@ -2193,7 +2235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>0</v>
       </c>
@@ -2216,7 +2258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>0</v>
       </c>
@@ -2239,7 +2281,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>0</v>
       </c>
@@ -2262,7 +2304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>0</v>
       </c>
@@ -2285,7 +2327,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>0</v>
       </c>
@@ -2308,7 +2350,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>0</v>
       </c>
@@ -2331,7 +2373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" t="str" cm="1">
         <f t="array" ref="A56:G66">[1]Context_Input!A68:G78</f>
         <v>#TemperatureSensor</v>
@@ -2355,7 +2397,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" t="str">
         <v>#TemperatureSensor</v>
       </c>
@@ -2378,7 +2420,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>0</v>
       </c>
@@ -2401,7 +2443,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>0</v>
       </c>
@@ -2424,7 +2466,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>0</v>
       </c>
@@ -2447,7 +2489,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>0</v>
       </c>
@@ -2470,7 +2512,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>0</v>
       </c>
@@ -2493,7 +2535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>0</v>
       </c>
@@ -2516,7 +2558,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>0</v>
       </c>
@@ -2539,7 +2581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>0</v>
       </c>
@@ -2562,7 +2604,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>0</v>
       </c>
@@ -2585,7 +2627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" t="str" cm="1">
         <f t="array" ref="A67:G77">[1]Context_Input!A81:G91</f>
         <v>#PressureSensor</v>
@@ -2609,7 +2651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" t="str">
         <v>#PressureSensor</v>
       </c>
@@ -2632,7 +2674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>0</v>
       </c>
@@ -2655,7 +2697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>0</v>
       </c>
@@ -2678,7 +2720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>0</v>
       </c>
@@ -2701,7 +2743,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>0</v>
       </c>
@@ -2724,7 +2766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>0</v>
       </c>
@@ -2747,7 +2789,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>0</v>
       </c>
@@ -2770,7 +2812,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>0</v>
       </c>
@@ -2793,7 +2835,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>0</v>
       </c>
@@ -2816,7 +2858,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>0</v>
       </c>
@@ -2839,7 +2881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" t="str" cm="1">
         <f t="array" ref="A78:G88">[1]Context_Input!A94:G104</f>
         <v>#MassFlowMeter</v>
@@ -2863,7 +2905,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" t="str">
         <v>#MassFlowMeter</v>
       </c>
@@ -2886,7 +2928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>0</v>
       </c>
@@ -2909,7 +2951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>0</v>
       </c>
@@ -2932,7 +2974,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>0</v>
       </c>
@@ -2955,7 +2997,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>0</v>
       </c>
@@ -2978,7 +3020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>0</v>
       </c>
@@ -3001,7 +3043,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>0</v>
       </c>
@@ -3024,7 +3066,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>0</v>
       </c>
@@ -3047,7 +3089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>0</v>
       </c>
@@ -3070,7 +3112,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>0</v>
       </c>
@@ -3093,7 +3135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" t="str" cm="1">
         <f t="array" ref="A89:G100">[1]Context_Input!A107:G118</f>
         <v>#Balance</v>
@@ -3101,8 +3143,8 @@
       <c r="B89" t="str">
         <v>#LastUsedPurpose_Balance_BeforeFirstUse</v>
       </c>
-      <c r="C89">
-        <v>0</v>
+      <c r="C89" t="str">
+        <v>#StartMassRDY</v>
       </c>
       <c r="D89" t="str">
         <v>#LastUsedTime_Balance</v>
@@ -3117,15 +3159,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" t="str">
         <v>#Balance</v>
       </c>
       <c r="B90" t="str">
         <v>#DigitalObjectID_Balance</v>
       </c>
-      <c r="C90">
-        <v>0</v>
+      <c r="C90" t="str">
+        <v>#FinalMass_RDY</v>
       </c>
       <c r="D90">
         <v>0</v>
@@ -3140,15 +3182,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>0</v>
       </c>
       <c r="B91">
         <v>0</v>
       </c>
-      <c r="C91">
-        <v>0</v>
+      <c r="C91" t="str">
+        <v>#FinalMass_RDEt</v>
       </c>
       <c r="D91">
         <v>0</v>
@@ -3163,15 +3205,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>0</v>
       </c>
       <c r="B92">
         <v>0</v>
       </c>
-      <c r="C92">
-        <v>0</v>
+      <c r="C92" t="str">
+        <v>#FinalMass_Dimer</v>
       </c>
       <c r="D92">
         <v>0</v>
@@ -3186,7 +3228,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>0</v>
       </c>
@@ -3209,7 +3251,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>0</v>
       </c>
@@ -3232,7 +3274,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>0</v>
       </c>
@@ -3255,7 +3297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>0</v>
       </c>
@@ -3278,7 +3320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>0</v>
       </c>
@@ -3301,7 +3343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>0</v>
       </c>
@@ -3324,7 +3366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>0</v>
       </c>
@@ -3347,7 +3389,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>0</v>
       </c>
@@ -3370,7 +3412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" t="str" cm="1">
         <f t="array" ref="A101:G111">[1]Context_Input!A124:G134</f>
         <v>#LiquidPhase</v>
@@ -3394,7 +3436,7 @@
         <v>#InitialMassFraction_Solvent_LiquidPhase</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" t="str">
         <v>#LiquidPhase</v>
       </c>
@@ -3417,7 +3459,7 @@
         <v>#InitialMassFraction_Water_LiquidPhase</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" t="str">
         <v>#LiquidPhase</v>
       </c>
@@ -3436,11 +3478,11 @@
       <c r="F103">
         <v>0</v>
       </c>
-      <c r="G103">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G103" t="str">
+        <v>#Reaction1</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" t="str">
         <v>#LiquidPhase</v>
       </c>
@@ -3459,11 +3501,11 @@
       <c r="F104">
         <v>0</v>
       </c>
-      <c r="G104">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G104" t="str">
+        <v>#Reaction2</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>0</v>
       </c>
@@ -3482,11 +3524,11 @@
       <c r="F105">
         <v>0</v>
       </c>
-      <c r="G105">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G105" t="str">
+        <v>#Reaction3</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>0</v>
       </c>
@@ -3509,7 +3551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>0</v>
       </c>
@@ -3532,7 +3574,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>0</v>
       </c>
@@ -3555,7 +3597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>0</v>
       </c>
@@ -3578,7 +3620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>0</v>
       </c>
@@ -3601,7 +3643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>0</v>
       </c>
@@ -3624,7 +3666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" t="str" cm="1">
         <f t="array" ref="A112:G122">[1]Context_Input!A137:G147</f>
         <v>#SolidPhase</v>
@@ -3648,7 +3690,7 @@
         <v>#RDY_Energy</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" t="str">
         <v>#SolidPhase</v>
       </c>
@@ -3667,11 +3709,11 @@
       <c r="F113">
         <v>0</v>
       </c>
-      <c r="G113">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G113" t="str">
+        <v>#Reaction1</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" t="str">
         <v>#SolidPhase</v>
       </c>
@@ -3694,7 +3736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>0</v>
       </c>
@@ -3717,7 +3759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>0</v>
       </c>
@@ -3740,7 +3782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>0</v>
       </c>
@@ -3763,7 +3805,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>0</v>
       </c>
@@ -3786,7 +3828,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>0</v>
       </c>
@@ -3809,7 +3851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>0</v>
       </c>
@@ -3832,7 +3874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>0</v>
       </c>
@@ -3855,7 +3897,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>0</v>
       </c>
@@ -3878,7 +3920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123" t="str" cm="1">
         <f t="array" ref="A123:G133">[1]Context_Input!A150:G160</f>
         <v>#CatalystPhase</v>
@@ -3898,11 +3940,11 @@
       <c r="F123">
         <v>0</v>
       </c>
-      <c r="G123">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G123" t="str">
+        <v>#Reaction1</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124" t="str">
         <v>#CatalystPhase</v>
       </c>
@@ -3921,11 +3963,11 @@
       <c r="F124">
         <v>0</v>
       </c>
-      <c r="G124">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G124" t="str">
+        <v>#Reaction2</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125" t="str">
         <v>#CatalystPhase</v>
       </c>
@@ -3944,11 +3986,11 @@
       <c r="F125">
         <v>0</v>
       </c>
-      <c r="G125">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G125" t="str">
+        <v>#Reaction3</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>0</v>
       </c>
@@ -3971,7 +4013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>0</v>
       </c>
@@ -3994,7 +4036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>0</v>
       </c>
@@ -4017,7 +4059,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>0</v>
       </c>
@@ -4040,7 +4082,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>0</v>
       </c>
@@ -4063,7 +4105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>0</v>
       </c>
@@ -4086,7 +4128,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>0</v>
       </c>
@@ -4109,7 +4151,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>0</v>
       </c>
@@ -4132,7 +4174,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A134" t="str" cm="1">
         <f t="array" ref="A134:G144">[1]Context_Input!A163:G173</f>
         <v>#GasPhase</v>
@@ -4156,7 +4198,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A135" t="str">
         <v>#GasPhase</v>
       </c>
@@ -4179,7 +4221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136" t="str">
         <v>#GasPhase</v>
       </c>
@@ -4202,7 +4244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>0</v>
       </c>
@@ -4225,7 +4267,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>0</v>
       </c>
@@ -4248,7 +4290,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>0</v>
       </c>
@@ -4271,7 +4313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>0</v>
       </c>
@@ -4294,7 +4336,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>0</v>
       </c>
@@ -4317,7 +4359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>0</v>
       </c>
@@ -4340,7 +4382,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>0</v>
       </c>
@@ -4363,7 +4405,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>0</v>
       </c>
@@ -4386,7 +4428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A145" t="str" cm="1">
         <f t="array" ref="A145:G155">[1]Context_Input!A176:G186</f>
         <v>#DispersedGasPhase</v>
@@ -4406,11 +4448,11 @@
       <c r="F145">
         <v>0</v>
       </c>
-      <c r="G145">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G145" t="str">
+        <v>#Reaction1</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A146" t="str">
         <v>#DispersedGasPhase</v>
       </c>
@@ -4433,7 +4475,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A147" t="str">
         <v>#DispersedGasPhase</v>
       </c>
@@ -4456,7 +4498,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>0</v>
       </c>
@@ -4479,7 +4521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>0</v>
       </c>
@@ -4502,7 +4544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>0</v>
       </c>
@@ -4525,7 +4567,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>0</v>
       </c>
@@ -4548,7 +4590,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>0</v>
       </c>
@@ -4571,7 +4613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>0</v>
       </c>
@@ -4594,7 +4636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>0</v>
       </c>
@@ -4617,7 +4659,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>0</v>
       </c>
@@ -4640,7 +4682,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A156" t="str" cm="1">
         <f t="array" ref="A156:G166">[1]Context_Input!A189:G199</f>
         <v>#CoolingFluidPhase</v>
@@ -4664,7 +4706,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A157" t="str">
         <v>#CoolingFluidPhase</v>
       </c>
@@ -4687,7 +4729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A158" t="str">
         <v>#CoolingFluidPhase</v>
       </c>
@@ -4710,7 +4752,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>0</v>
       </c>
@@ -4733,7 +4775,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>0</v>
       </c>
@@ -4756,7 +4798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>0</v>
       </c>
@@ -4779,7 +4821,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>0</v>
       </c>
@@ -4802,7 +4844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>0</v>
       </c>
@@ -4825,7 +4867,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>0</v>
       </c>
@@ -4848,7 +4890,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>0</v>
       </c>
@@ -4871,7 +4913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>0</v>
       </c>
@@ -4894,7 +4936,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A167" t="str" cm="1">
         <f t="array" ref="A167:G177">[1]Context_Input!A202:G212</f>
         <v>#HydrogenSpargerPhase</v>
@@ -4918,7 +4960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A168" t="str">
         <v>#HydrogenSpargerPhase</v>
       </c>
@@ -4941,7 +4983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A169" t="str">
         <v>#HydrogenSpargerPhase</v>
       </c>
@@ -4964,7 +5006,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>0</v>
       </c>
@@ -4987,7 +5029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>0</v>
       </c>
@@ -5010,7 +5052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>0</v>
       </c>
@@ -5033,7 +5075,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A173">
         <v>0</v>
       </c>
@@ -5056,7 +5098,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A174">
         <v>0</v>
       </c>
@@ -5079,7 +5121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A175">
         <v>0</v>
       </c>
@@ -5102,7 +5144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A176">
         <v>0</v>
       </c>
@@ -5125,7 +5167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>0</v>
       </c>
@@ -5148,7 +5190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A178" t="str" cm="1">
         <f t="array" ref="A178:G188">[1]Context_Input!A215:G225</f>
         <v>#CleaningFluidPhase</v>
@@ -5172,7 +5214,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>0</v>
       </c>
@@ -5195,7 +5237,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>0</v>
       </c>
@@ -5218,7 +5260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>0</v>
       </c>
@@ -5241,7 +5283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>0</v>
       </c>
@@ -5264,7 +5306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A183">
         <v>0</v>
       </c>
@@ -5287,7 +5329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>0</v>
       </c>
@@ -5310,7 +5352,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A185">
         <v>0</v>
       </c>
@@ -5333,7 +5375,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>0</v>
       </c>
@@ -5356,7 +5398,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A187">
         <v>0</v>
       </c>
@@ -5379,7 +5421,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A188">
         <v>0</v>
       </c>
@@ -5402,7 +5444,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A189" t="str" cm="1">
         <f t="array" ref="A189:G199">[1]Context_Input!A231:G241</f>
         <v>#H2</v>
@@ -5426,7 +5468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A190" t="str">
         <v>#H2</v>
       </c>
@@ -5449,7 +5491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A191" t="str">
         <v>#H2</v>
       </c>
@@ -5472,7 +5514,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>0</v>
       </c>
@@ -5495,7 +5537,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>0</v>
       </c>
@@ -5518,7 +5560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A194">
         <v>0</v>
       </c>
@@ -5541,7 +5583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A195">
         <v>0</v>
       </c>
@@ -5564,7 +5606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A196">
         <v>0</v>
       </c>
@@ -5587,7 +5629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A197">
         <v>0</v>
       </c>
@@ -5610,7 +5652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A198">
         <v>0</v>
       </c>
@@ -5633,7 +5675,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A199">
         <v>0</v>
       </c>
@@ -5656,7 +5698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A200" t="str" cm="1">
         <f t="array" ref="A200:G210">[1]Context_Input!A244:G254</f>
         <v>#H2O</v>
@@ -5680,7 +5722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A201">
         <v>0</v>
       </c>
@@ -5703,7 +5745,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A202">
         <v>0</v>
       </c>
@@ -5726,7 +5768,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A203">
         <v>0</v>
       </c>
@@ -5749,7 +5791,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A204">
         <v>0</v>
       </c>
@@ -5772,7 +5814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A205">
         <v>0</v>
       </c>
@@ -5795,7 +5837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A206">
         <v>0</v>
       </c>
@@ -5818,7 +5860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A207">
         <v>0</v>
       </c>
@@ -5841,7 +5883,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A208">
         <v>0</v>
       </c>
@@ -5864,7 +5906,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A209">
         <v>0</v>
       </c>
@@ -5887,7 +5929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A210">
         <v>0</v>
       </c>
@@ -5910,7 +5952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A211" t="str" cm="1">
         <f t="array" ref="A211:G221">[1]Context_Input!A257:G267</f>
         <v>#Solvent</v>
@@ -5934,7 +5976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A212">
         <v>0</v>
       </c>
@@ -5957,7 +5999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A213">
         <v>0</v>
       </c>
@@ -5980,7 +6022,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A214">
         <v>0</v>
       </c>
@@ -6003,7 +6045,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A215">
         <v>0</v>
       </c>
@@ -6026,7 +6068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A216">
         <v>0</v>
       </c>
@@ -6049,7 +6091,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A217">
         <v>0</v>
       </c>
@@ -6072,7 +6114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A218">
         <v>0</v>
       </c>
@@ -6095,7 +6137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A219">
         <v>0</v>
       </c>
@@ -6118,7 +6160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A220">
         <v>0</v>
       </c>
@@ -6141,7 +6183,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A221">
         <v>0</v>
       </c>
@@ -6164,7 +6206,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A222" t="str" cm="1">
         <f t="array" ref="A222:G232">[1]Context_Input!A270:G280</f>
         <v>#RDY</v>
@@ -6188,7 +6230,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A223" t="str">
         <v>#RDY</v>
       </c>
@@ -6211,7 +6253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A224" t="str">
         <v>#RDY</v>
       </c>
@@ -6234,7 +6276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A225">
         <v>0</v>
       </c>
@@ -6257,7 +6299,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A226">
         <v>0</v>
       </c>
@@ -6280,7 +6322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A227">
         <v>0</v>
       </c>
@@ -6303,7 +6345,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A228">
         <v>0</v>
       </c>
@@ -6326,7 +6368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A229">
         <v>0</v>
       </c>
@@ -6349,7 +6391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="230" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A230">
         <v>0</v>
       </c>
@@ -6372,7 +6414,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="231" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A231">
         <v>0</v>
       </c>
@@ -6395,7 +6437,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="232" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A232">
         <v>0</v>
       </c>
@@ -6418,7 +6460,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="233" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A233" cm="1">
         <f t="array" ref="A233:G243">[1]Context_Input!A283:G293</f>
         <v>0</v>
@@ -6442,7 +6484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="234" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A234">
         <v>0</v>
       </c>
@@ -6465,7 +6507,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="235" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A235">
         <v>0</v>
       </c>
@@ -6488,7 +6530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="236" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A236">
         <v>0</v>
       </c>
@@ -6511,7 +6553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="237" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A237">
         <v>0</v>
       </c>
@@ -6534,7 +6576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="238" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A238">
         <v>0</v>
       </c>
@@ -6557,7 +6599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="239" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A239">
         <v>0</v>
       </c>
@@ -6580,7 +6622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="240" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A240">
         <v>0</v>
       </c>
@@ -6603,7 +6645,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="241" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A241">
         <v>0</v>
       </c>
@@ -6626,7 +6668,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="242" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A242">
         <v>0</v>
       </c>
@@ -6649,7 +6691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="243" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A243">
         <v>0</v>
       </c>
@@ -6672,7 +6714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="244" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A244" cm="1">
         <f t="array" ref="A244:G254">[1]Context_Input!A296:G306</f>
         <v>0</v>
@@ -6696,7 +6738,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="245" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A245">
         <v>0</v>
       </c>
@@ -6719,7 +6761,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="246" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A246">
         <v>0</v>
       </c>
@@ -6742,7 +6784,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="247" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A247">
         <v>0</v>
       </c>
@@ -6765,7 +6807,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A248">
         <v>0</v>
       </c>
@@ -6788,7 +6830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="249" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A249">
         <v>0</v>
       </c>
@@ -6811,7 +6853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="250" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A250">
         <v>0</v>
       </c>
@@ -6834,7 +6876,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="251" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A251">
         <v>0</v>
       </c>
@@ -6857,7 +6899,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="252" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A252">
         <v>0</v>
       </c>
@@ -6880,7 +6922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="253" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A253">
         <v>0</v>
       </c>
@@ -6903,7 +6945,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="254" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A254">
         <v>0</v>
       </c>
@@ -6926,7 +6968,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="255" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A255" cm="1">
         <f t="array" ref="A255:G265">[1]Context_Input!A309:G319</f>
         <v>0</v>
@@ -6950,7 +6992,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="256" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A256">
         <v>0</v>
       </c>
@@ -6973,7 +7015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="257" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A257">
         <v>0</v>
       </c>
@@ -6996,7 +7038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="258" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A258">
         <v>0</v>
       </c>
@@ -7019,7 +7061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="259" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A259">
         <v>0</v>
       </c>
@@ -7042,7 +7084,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="260" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A260">
         <v>0</v>
       </c>
@@ -7065,7 +7107,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="261" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A261">
         <v>0</v>
       </c>
@@ -7088,7 +7130,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="262" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A262">
         <v>0</v>
       </c>
@@ -7111,7 +7153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="263" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A263">
         <v>0</v>
       </c>
@@ -7134,7 +7176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="264" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A264">
         <v>0</v>
       </c>
@@ -7157,7 +7199,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="265" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A265">
         <v>0</v>
       </c>
@@ -7180,7 +7222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="266" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A266" t="str" cm="1">
         <f t="array" ref="A266:G276">[1]Context_Input!A322:G332</f>
         <v>#RDEt</v>
@@ -7204,7 +7246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="267" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A267">
         <v>0</v>
       </c>
@@ -7227,7 +7269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="268" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A268">
         <v>0</v>
       </c>
@@ -7250,7 +7292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="269" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A269">
         <v>0</v>
       </c>
@@ -7273,7 +7315,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="270" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A270">
         <v>0</v>
       </c>
@@ -7296,7 +7338,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="271" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A271">
         <v>0</v>
       </c>
@@ -7319,7 +7361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="272" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A272">
         <v>0</v>
       </c>
@@ -7342,7 +7384,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="273" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A273">
         <v>0</v>
       </c>
@@ -7365,7 +7407,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="274" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A274">
         <v>0</v>
       </c>
@@ -7388,7 +7430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="275" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A275">
         <v>0</v>
       </c>
@@ -7411,7 +7453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="276" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A276">
         <v>0</v>
       </c>
@@ -7434,7 +7476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="277" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A277" t="str" cm="1">
         <f t="array" ref="A277:G287">[1]Context_Input!A335:G345</f>
         <v>#Dimer1</v>
@@ -7458,7 +7500,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="278" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A278">
         <v>0</v>
       </c>
@@ -7481,7 +7523,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="279" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A279">
         <v>0</v>
       </c>
@@ -7504,7 +7546,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="280" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A280">
         <v>0</v>
       </c>
@@ -7527,7 +7569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="281" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A281">
         <v>0</v>
       </c>
@@ -7550,7 +7592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="282" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A282">
         <v>0</v>
       </c>
@@ -7573,7 +7615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="283" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A283">
         <v>0</v>
       </c>
@@ -7596,7 +7638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="284" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A284">
         <v>0</v>
       </c>
@@ -7619,7 +7661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="285" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A285">
         <v>0</v>
       </c>
@@ -7642,7 +7684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="286" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A286">
         <v>0</v>
       </c>
@@ -7665,7 +7707,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="287" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A287">
         <v>0</v>
       </c>
@@ -7688,7 +7730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="288" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A288" t="str" cm="1">
         <f t="array" ref="A288:G298">[1]Context_Input!A348:G358</f>
         <v>#Dimer2</v>
@@ -7712,7 +7754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="289" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A289">
         <v>0</v>
       </c>
@@ -7735,7 +7777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="290" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A290">
         <v>0</v>
       </c>
@@ -7758,7 +7800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="291" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A291">
         <v>0</v>
       </c>
@@ -7781,7 +7823,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="292" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A292">
         <v>0</v>
       </c>
@@ -7804,7 +7846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="293" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A293">
         <v>0</v>
       </c>
@@ -7827,7 +7869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="294" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A294">
         <v>0</v>
       </c>
@@ -7850,7 +7892,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="295" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A295">
         <v>0</v>
       </c>
@@ -7873,7 +7915,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="296" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A296">
         <v>0</v>
       </c>
@@ -7896,7 +7938,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="297" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A297">
         <v>0</v>
       </c>
@@ -7919,7 +7961,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="298" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A298">
         <v>0</v>
       </c>
@@ -7942,7 +7984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="299" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A299" t="str" cm="1">
         <f t="array" ref="A299:G309">[1]Context_Input!A361:G371</f>
         <v>#Pt</v>
@@ -7966,7 +8008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="300" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A300">
         <v>0</v>
       </c>
@@ -7989,7 +8031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="301" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A301">
         <v>0</v>
       </c>
@@ -8012,7 +8054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="302" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A302">
         <v>0</v>
       </c>
@@ -8035,7 +8077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="303" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A303">
         <v>0</v>
       </c>
@@ -8058,7 +8100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="304" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A304">
         <v>0</v>
       </c>
@@ -8081,7 +8123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="305" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A305">
         <v>0</v>
       </c>
@@ -8104,7 +8146,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="306" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A306">
         <v>0</v>
       </c>
@@ -8127,7 +8169,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="307" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A307">
         <v>0</v>
       </c>
@@ -8150,7 +8192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="308" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A308">
         <v>0</v>
       </c>
@@ -8173,7 +8215,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="309" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A309">
         <v>0</v>
       </c>

</xml_diff>